<commit_message>
update files, rename folders, minor bot changes
</commit_message>
<xml_diff>
--- a/core-extensions/SabberStoneCoreAi/my_results/experiments-analysis.xlsx
+++ b/core-extensions/SabberStoneCoreAi/my_results/experiments-analysis.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pics_Movies\vids\PWr\Sem10\magisterka\SabberStone\core-extensions\SabberStoneCoreAi\my_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA907C3-9EAB-4119-BEB4-26921B026DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3422C5CB-5D8D-4A1C-8A7E-004F838E9E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3405" yWindow="1395" windowWidth="28800" windowHeight="15885" xr2:uid="{23FC15A1-DE11-4199-B1D8-4DE8B55B0A24}"/>
+    <workbookView xWindow="2400" yWindow="2790" windowWidth="28800" windowHeight="15885" activeTab="1" xr2:uid="{23FC15A1-DE11-4199-B1D8-4DE8B55B0A24}"/>
   </bookViews>
   <sheets>
     <sheet name="Weights" sheetId="1" r:id="rId1"/>
-    <sheet name="Fights" sheetId="2" r:id="rId2"/>
+    <sheet name="Fights_8_8_200" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="112">
   <si>
     <t>Hero Health Reduced</t>
   </si>
@@ -256,12 +256,6 @@
     <t>p2 wins</t>
   </si>
   <si>
-    <t>base-8-8-200</t>
-  </si>
-  <si>
-    <t>63-8-8-200</t>
-  </si>
-  <si>
     <t>p1 wins</t>
   </si>
   <si>
@@ -277,18 +271,9 @@
     <t>p2winrate</t>
   </si>
   <si>
-    <t>28-8-8-200</t>
-  </si>
-  <si>
     <t>base</t>
   </si>
   <si>
-    <t>21d</t>
-  </si>
-  <si>
-    <t>21d(base-weights)-8-8-200</t>
-  </si>
-  <si>
     <t>WinAvgTrn</t>
   </si>
   <si>
@@ -307,16 +292,109 @@
     <t>Modified - 63 smooth parameters</t>
   </si>
   <si>
-    <t>21Normalized</t>
-  </si>
-  <si>
-    <t>0.5018309634301501, 0.7423451363740952, 0.0, 1.0, 0.7889671898460878, 1.0, 0.5801904002480903, 0.0, 0.26450840963181244, 0.49188495725867865, 0.4170883075336374, 0.09983441078009811, 0.3125999621707864, 1.0, 0.0, 0.27976033425320757, 0.469499077972434, 0.5111432760491664, 0.30663855232489895, 0.7040165654971762, 0.3471960774301261, 0.47628480507854354, 0.8423451363740951, 0.014705895432485551, 0.9956599374568458, 0.7078432854533878, 1.0, 0.48019040024809034, 0.013677038307942603, 0.16450840963181243, 0.4623716489913056, 0.31708830753363737, 0.0, 0.34874940380617453, 0.9, 0.03904821528201339, 0.22196476903852289, 0.569499077972434, 0.5470182144844639, 0.32445682580715235, 0.6040165654971762, 0.2471960774301261, 0.5728993986822584, 0.9423451363740951, 0.08947250274492421, 1.0, 0.6466465957242477, 1.0, 0.5074274005848062, 0.0, 0.14289177800553857, 0.5623716489913057, 0.24690025994053244, 0.0, 0.30105336034734864, 0.9065068994520135, 0.0, 0.26961343445188857, 0.5041212070306388, 0.48225812616933666, 0.4244568258071524, 0.5040165654971762, 0.31869428836394775</t>
-  </si>
-  <si>
     <t>Column1</t>
   </si>
   <si>
     <t>Column2</t>
+  </si>
+  <si>
+    <t>28Normalized</t>
+  </si>
+  <si>
+    <t>0.4489769376909381, 1, 0, 0.2200813583097922, 0.36904127870754105, 0.5734997567308384, 0.7609641739977115, 0, 1, 1, 0.8855302018224294, 0.8306653004086676, 0.5377170358339709, 0.6550543815442608, 0.2772477549959537, 0.9592308396183514, 0, 0.24293859078887203, 0.2529414637771258, 0.9405997864481604, 0, 0.8282849886177859, 0.7886381793044395, 0.24788606446216535, 0.4452603904961968, 0.8513638103721802, 0.09766786771815637, 0.4317827066736215, 0.38365795363489325, 0.4474496490628219, 0.8204377341428768, 0.17300304887729573, 0.33618881620573426, 0.07601503063487242, 0.09118924302373758, 0.5503333105413887, 1.317969980390527, 0.6145414649828274, 0.3519713726795352, 0.2963622514040038, 0.276955383826611, 0.8005728430930316, 0.02427733053940036, 1.6067053727056138, 0.4862103185448709, 0.10861069729595417, 0.29557917692469254, 0.8715150786731626, 0.839398210617237, 0.6870816863298209, 0.6557872328730052, 0.13697399763482626, 0.16569205613001692, 0.7745538427122949, 0.2968141695339541, 1.5314411976433369</t>
+  </si>
+  <si>
+    <t>0.4489769376909381</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.2200813583097922</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.36904127870754105</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.5734997567308384</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.7609641739977115</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.8855302018224294</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.8306653004086676</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.5377170358339709</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.6550543815442608</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.2772477549959537</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.9592308396183514</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.24293859078887203</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.2529414637771258</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.9405997864481604</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.8282849886177859</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.7886381793044395</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.24788606446216535</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.4452603904961968</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.8513638103721802</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.09766786771815637</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.4317827066736215</t>
+  </si>
+  <si>
+    <t>21depth</t>
+  </si>
+  <si>
+    <t>63 smooth</t>
+  </si>
+  <si>
+    <t>28 normalized</t>
+  </si>
+  <si>
+    <t>0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126</t>
+  </si>
+  <si>
+    <t>0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0</t>
+  </si>
+  <si>
+    <t>0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108</t>
+  </si>
+  <si>
+    <t>0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126#0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0#0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108</t>
+  </si>
+  <si>
+    <t>21d(base-weights)</t>
+  </si>
+  <si>
+    <t>21d(learned)</t>
+  </si>
+  <si>
+    <t>28Normalized(fix score minion)</t>
   </si>
 </sst>
 </file>
@@ -375,7 +453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -389,7 +467,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,8 +643,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4F7477B9-42AA-4499-B8FA-2A689B22B5B7}" name="Table36359" displayName="Table36359" ref="BY31:CG53" totalsRowShown="0">
-  <autoFilter ref="BY31:CG53" xr:uid="{4F7477B9-42AA-4499-B8FA-2A689B22B5B7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4F7477B9-42AA-4499-B8FA-2A689B22B5B7}" name="Table36359" displayName="Table36359" ref="BY31:CG60" totalsRowShown="0">
+  <autoFilter ref="BY31:CG60" xr:uid="{4F7477B9-42AA-4499-B8FA-2A689B22B5B7}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{4DD5DEC6-A376-4203-AD7B-42CE5CBAE520}" name="NUM_GAMES"/>
     <tableColumn id="2" xr3:uid="{0372BE09-D705-4AF9-8CC0-7773767B0E9A}" name="POP_SIZE"/>
@@ -902,7 +979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{719E6D9B-34F9-44C1-9C05-29B97EE9AFF1}">
-  <dimension ref="A1:CJ127"/>
+  <dimension ref="A1:CG127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="5.7109375" customWidth="1"/>
@@ -942,6 +1019,7 @@
     <col min="58" max="58" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="59" max="59" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.140625" customWidth="1"/>
     <col min="66" max="66" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="12.85546875" customWidth="1"/>
     <col min="68" max="68" width="13.85546875" customWidth="1"/>
@@ -1716,7 +1794,7 @@
       <c r="AT29" s="8"/>
       <c r="AU29" s="8"/>
       <c r="AY29" s="8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="AZ29" s="8"/>
       <c r="BA29" s="8"/>
@@ -1727,7 +1805,7 @@
       <c r="BF29" s="8"/>
       <c r="BG29" s="8"/>
       <c r="BK29" s="8" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="BL29" s="8"/>
       <c r="BM29" s="8"/>
@@ -1740,7 +1818,7 @@
       <c r="BT29" s="8"/>
       <c r="BU29" s="8"/>
       <c r="BY29" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="BZ29" s="8"/>
       <c r="CA29" s="8"/>
@@ -1967,10 +2045,10 @@
         <v>24</v>
       </c>
       <c r="BO31" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="BP31" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="BQ31" t="s">
         <v>25</v>
@@ -2164,7 +2242,7 @@
         <v>595</v>
       </c>
       <c r="BT32">
-        <v>301</v>
+        <v>601.25</v>
       </c>
       <c r="BU32">
         <v>14.4</v>
@@ -2182,8 +2260,23 @@
         <f>BY32*(2*BZ32-1)*9</f>
         <v>1080</v>
       </c>
-    </row>
-    <row r="33" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="CC32">
+        <v>630</v>
+      </c>
+      <c r="CD32">
+        <v>719</v>
+      </c>
+      <c r="CE32">
+        <v>680</v>
+      </c>
+      <c r="CF32">
+        <v>671</v>
+      </c>
+      <c r="CG32">
+        <v>31.3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -2273,22 +2366,22 @@
       <c r="BJ33">
         <v>1</v>
       </c>
-      <c r="BK33" s="9">
+      <c r="BK33">
         <v>0.50183096343014999</v>
       </c>
-      <c r="BL33" s="9">
+      <c r="BL33">
         <v>0.37226920824196702</v>
       </c>
-      <c r="BM33" s="9">
+      <c r="BM33">
         <v>0.98307296801857402</v>
       </c>
-      <c r="BN33" s="9">
+      <c r="BN33">
         <v>0.50183096343014999</v>
       </c>
-      <c r="BO33" s="9">
+      <c r="BO33">
         <v>0.47628480507854298</v>
       </c>
-      <c r="BP33" s="9">
+      <c r="BP33">
         <v>0.57289939868225803</v>
       </c>
       <c r="BQ33">
@@ -2305,7 +2398,7 @@
       </c>
       <c r="BT33">
         <f>BT32/$AD$32</f>
-        <v>0.27870370370370373</v>
+        <v>0.55671296296296291</v>
       </c>
       <c r="BW33" t="s">
         <v>0</v>
@@ -2313,8 +2406,27 @@
       <c r="BX33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY33" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC33">
+        <f>CC32/$AD$32</f>
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="CD33">
+        <f t="shared" ref="CD33:CF33" si="0">CD32/$AD$32</f>
+        <v>0.66574074074074074</v>
+      </c>
+      <c r="CE33">
+        <f t="shared" si="0"/>
+        <v>0.62962962962962965</v>
+      </c>
+      <c r="CF33">
+        <f t="shared" si="0"/>
+        <v>0.62129629629629635</v>
+      </c>
+    </row>
+    <row r="34" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
@@ -2372,22 +2484,22 @@
       <c r="BJ34">
         <v>2</v>
       </c>
-      <c r="BK34" s="9">
+      <c r="BK34">
         <v>0.74234513637409505</v>
       </c>
-      <c r="BL34" s="9">
-        <v>1</v>
-      </c>
-      <c r="BM34" s="9">
-        <v>1</v>
-      </c>
-      <c r="BN34" s="9">
+      <c r="BL34">
+        <v>1</v>
+      </c>
+      <c r="BM34">
+        <v>1</v>
+      </c>
+      <c r="BN34">
         <v>0.74234513637409505</v>
       </c>
-      <c r="BO34" s="9">
+      <c r="BO34">
         <v>0.84234513637409503</v>
       </c>
-      <c r="BP34" s="9">
+      <c r="BP34">
         <v>0.942345136374095</v>
       </c>
       <c r="BW34" t="s">
@@ -2396,8 +2508,11 @@
       <c r="BX34">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -2455,22 +2570,22 @@
       <c r="BJ35">
         <v>3</v>
       </c>
-      <c r="BK35" s="9">
-        <v>0</v>
-      </c>
-      <c r="BL35" s="9">
+      <c r="BK35">
+        <v>0</v>
+      </c>
+      <c r="BL35">
         <v>0.57352947716242697</v>
       </c>
-      <c r="BM35" s="9">
+      <c r="BM35">
         <v>0.87383303656219302</v>
       </c>
-      <c r="BN35" s="9">
-        <v>0</v>
-      </c>
-      <c r="BO35" s="9">
+      <c r="BN35">
+        <v>0</v>
+      </c>
+      <c r="BO35">
         <v>1.4705895432485501E-2</v>
       </c>
-      <c r="BP35" s="9">
+      <c r="BP35">
         <v>8.9472502744924201E-2</v>
       </c>
       <c r="BW35" t="s">
@@ -2479,8 +2594,11 @@
       <c r="BX35">
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -2538,22 +2656,22 @@
       <c r="BJ36">
         <v>4</v>
       </c>
-      <c r="BK36" s="9">
-        <v>1</v>
-      </c>
-      <c r="BL36" s="9">
+      <c r="BK36">
+        <v>1</v>
+      </c>
+      <c r="BL36">
         <v>0.478299687284229</v>
       </c>
-      <c r="BM36" s="9">
+      <c r="BM36">
         <v>0.57748137724547399</v>
       </c>
-      <c r="BN36" s="9">
-        <v>1</v>
-      </c>
-      <c r="BO36" s="9">
+      <c r="BN36">
+        <v>1</v>
+      </c>
+      <c r="BO36">
         <v>0.995659937456845</v>
       </c>
-      <c r="BP36" s="9">
+      <c r="BP36">
         <v>1</v>
       </c>
       <c r="BW36" t="s">
@@ -2562,8 +2680,11 @@
       <c r="BX36">
         <v>4</v>
       </c>
-    </row>
-    <row r="37" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY36" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="37" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -2621,22 +2742,22 @@
       <c r="BJ37">
         <v>5</v>
       </c>
-      <c r="BK37" s="9">
+      <c r="BK37">
         <v>0.78896718984608705</v>
       </c>
-      <c r="BL37" s="9">
+      <c r="BL37">
         <v>9.4380478036499696E-2</v>
       </c>
-      <c r="BM37" s="9">
+      <c r="BM37">
         <v>0.19401655135429899</v>
       </c>
-      <c r="BN37" s="9">
+      <c r="BN37">
         <v>0.78896718984608705</v>
       </c>
-      <c r="BO37" s="9">
+      <c r="BO37">
         <v>0.70784328545338704</v>
       </c>
-      <c r="BP37" s="9">
+      <c r="BP37">
         <v>0.64664659572424699</v>
       </c>
       <c r="BW37" t="s">
@@ -2645,8 +2766,11 @@
       <c r="BX37">
         <v>5</v>
       </c>
-    </row>
-    <row r="38" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY37" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -2704,22 +2828,22 @@
       <c r="BJ38">
         <v>6</v>
       </c>
-      <c r="BK38" s="9">
-        <v>1</v>
-      </c>
-      <c r="BL38" s="9">
-        <v>1</v>
-      </c>
-      <c r="BM38" s="9">
-        <v>1</v>
-      </c>
-      <c r="BN38" s="9">
-        <v>1</v>
-      </c>
-      <c r="BO38" s="9">
-        <v>1</v>
-      </c>
-      <c r="BP38" s="9">
+      <c r="BK38">
+        <v>1</v>
+      </c>
+      <c r="BL38">
+        <v>1</v>
+      </c>
+      <c r="BM38">
+        <v>1</v>
+      </c>
+      <c r="BN38">
+        <v>1</v>
+      </c>
+      <c r="BO38">
+        <v>1</v>
+      </c>
+      <c r="BP38">
         <v>1</v>
       </c>
       <c r="BW38" t="s">
@@ -2728,8 +2852,11 @@
       <c r="BX38">
         <v>6</v>
       </c>
-    </row>
-    <row r="39" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY38" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -2787,22 +2914,22 @@
       <c r="BJ39">
         <v>7</v>
       </c>
-      <c r="BK39" s="9">
+      <c r="BK39">
         <v>0.58019040024808999</v>
       </c>
-      <c r="BL39" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM39" s="9">
+      <c r="BL39">
+        <v>0</v>
+      </c>
+      <c r="BM39">
         <v>0.63618500168357905</v>
       </c>
-      <c r="BN39" s="9">
+      <c r="BN39">
         <v>0.58019040024808999</v>
       </c>
-      <c r="BO39" s="9">
+      <c r="BO39">
         <v>0.48019040024809001</v>
       </c>
-      <c r="BP39" s="9">
+      <c r="BP39">
         <v>0.50742740058480595</v>
       </c>
       <c r="BW39" t="s">
@@ -2811,8 +2938,11 @@
       <c r="BX39">
         <v>7</v>
       </c>
-    </row>
-    <row r="40" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY39" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>7</v>
       </c>
@@ -2870,22 +3000,22 @@
       <c r="BJ40">
         <v>8</v>
       </c>
-      <c r="BK40" s="9">
-        <v>0</v>
-      </c>
-      <c r="BL40" s="9">
+      <c r="BK40">
+        <v>0</v>
+      </c>
+      <c r="BL40">
         <v>0.56838519153971301</v>
       </c>
-      <c r="BM40" s="9">
-        <v>0</v>
-      </c>
-      <c r="BN40" s="9">
-        <v>0</v>
-      </c>
-      <c r="BO40" s="9">
+      <c r="BM40">
+        <v>0</v>
+      </c>
+      <c r="BN40">
+        <v>0</v>
+      </c>
+      <c r="BO40">
         <v>1.3677038307942599E-2</v>
       </c>
-      <c r="BP40" s="9">
+      <c r="BP40">
         <v>0</v>
       </c>
       <c r="BW40" t="s">
@@ -2894,8 +3024,11 @@
       <c r="BX40">
         <v>8</v>
       </c>
-    </row>
-    <row r="41" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY40" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -2953,22 +3086,22 @@
       <c r="BJ41">
         <v>9</v>
       </c>
-      <c r="BK41" s="9">
+      <c r="BK41">
         <v>0.26450840963181199</v>
       </c>
-      <c r="BL41" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM41" s="9">
+      <c r="BL41">
+        <v>0</v>
+      </c>
+      <c r="BM41">
         <v>0.39191684186863002</v>
       </c>
-      <c r="BN41" s="9">
+      <c r="BN41">
         <v>0.26450840963181199</v>
       </c>
-      <c r="BO41" s="9">
+      <c r="BO41">
         <v>0.16450840963181201</v>
       </c>
-      <c r="BP41" s="9">
+      <c r="BP41">
         <v>0.14289177800553801</v>
       </c>
       <c r="BW41" t="s">
@@ -2977,8 +3110,11 @@
       <c r="BX41">
         <v>9</v>
       </c>
-    </row>
-    <row r="42" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY41" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -3036,22 +3172,22 @@
       <c r="BJ42">
         <v>10</v>
       </c>
-      <c r="BK42" s="9">
+      <c r="BK42">
         <v>0.49188495725867798</v>
       </c>
-      <c r="BL42" s="9">
+      <c r="BL42">
         <v>0.35243345866313402</v>
       </c>
-      <c r="BM42" s="9">
-        <v>1</v>
-      </c>
-      <c r="BN42" s="9">
+      <c r="BM42">
+        <v>1</v>
+      </c>
+      <c r="BN42">
         <v>0.49188495725867798</v>
       </c>
-      <c r="BO42" s="9">
+      <c r="BO42">
         <v>0.46237164899130501</v>
       </c>
-      <c r="BP42" s="9">
+      <c r="BP42">
         <v>0.56237164899130498</v>
       </c>
       <c r="BW42" t="s">
@@ -3060,8 +3196,11 @@
       <c r="BX42">
         <v>10</v>
       </c>
-    </row>
-    <row r="43" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY42" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -3119,22 +3258,22 @@
       <c r="BJ43">
         <v>11</v>
       </c>
-      <c r="BK43" s="9">
+      <c r="BK43">
         <v>0.41708830753363701</v>
       </c>
-      <c r="BL43" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM43" s="9">
+      <c r="BL43">
+        <v>0</v>
+      </c>
+      <c r="BM43">
         <v>0.14905976203447499</v>
       </c>
-      <c r="BN43" s="9">
+      <c r="BN43">
         <v>0.41708830753363701</v>
       </c>
-      <c r="BO43" s="9">
+      <c r="BO43">
         <v>0.31708830753363698</v>
       </c>
-      <c r="BP43" s="9">
+      <c r="BP43">
         <v>0.246900259940532</v>
       </c>
       <c r="BW43" t="s">
@@ -3143,8 +3282,11 @@
       <c r="BX43">
         <v>11</v>
       </c>
-    </row>
-    <row r="44" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY43" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -3202,22 +3344,22 @@
       <c r="BJ44">
         <v>12</v>
       </c>
-      <c r="BK44" s="9">
+      <c r="BK44">
         <v>9.9834410780098096E-2</v>
       </c>
-      <c r="BL44" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM44" s="9">
-        <v>0</v>
-      </c>
-      <c r="BN44" s="9">
+      <c r="BL44">
+        <v>0</v>
+      </c>
+      <c r="BM44">
+        <v>0</v>
+      </c>
+      <c r="BN44">
         <v>9.9834410780098096E-2</v>
       </c>
-      <c r="BO44" s="9">
-        <v>0</v>
-      </c>
-      <c r="BP44" s="9">
+      <c r="BO44">
+        <v>0</v>
+      </c>
+      <c r="BP44">
         <v>0</v>
       </c>
       <c r="BW44" t="s">
@@ -3226,8 +3368,11 @@
       <c r="BX44">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY44" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -3285,22 +3430,22 @@
       <c r="BJ45">
         <v>13</v>
       </c>
-      <c r="BK45" s="9">
+      <c r="BK45">
         <v>0.31259996217078601</v>
       </c>
-      <c r="BL45" s="9">
+      <c r="BL45">
         <v>0.68074720817694001</v>
       </c>
-      <c r="BM45" s="9">
+      <c r="BM45">
         <v>0.26151978270587001</v>
       </c>
-      <c r="BN45" s="9">
+      <c r="BN45">
         <v>0.31259996217078601</v>
       </c>
-      <c r="BO45" s="9">
+      <c r="BO45">
         <v>0.34874940380617397</v>
       </c>
-      <c r="BP45" s="9">
+      <c r="BP45">
         <v>0.30105336034734798</v>
       </c>
       <c r="BW45" t="s">
@@ -3309,8 +3454,11 @@
       <c r="BX45">
         <v>13</v>
       </c>
-    </row>
-    <row r="46" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY45" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="46" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -3368,22 +3516,22 @@
       <c r="BJ46">
         <v>14</v>
       </c>
-      <c r="BK46" s="9">
-        <v>1</v>
-      </c>
-      <c r="BL46" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM46" s="9">
+      <c r="BK46">
+        <v>1</v>
+      </c>
+      <c r="BL46">
+        <v>0</v>
+      </c>
+      <c r="BM46">
         <v>0.53253449726006696</v>
       </c>
-      <c r="BN46" s="9">
-        <v>1</v>
-      </c>
-      <c r="BO46" s="9">
+      <c r="BN46">
+        <v>1</v>
+      </c>
+      <c r="BO46">
         <v>0.9</v>
       </c>
-      <c r="BP46" s="9">
+      <c r="BP46">
         <v>0.90650689945201302</v>
       </c>
       <c r="BW46" t="s">
@@ -3392,8 +3540,11 @@
       <c r="BX46">
         <v>14</v>
       </c>
-    </row>
-    <row r="47" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY46" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -3451,22 +3602,22 @@
       <c r="BJ47">
         <v>15</v>
       </c>
-      <c r="BK47" s="9">
-        <v>0</v>
-      </c>
-      <c r="BL47" s="9">
+      <c r="BK47">
+        <v>0</v>
+      </c>
+      <c r="BL47">
         <v>0.69524107641006605</v>
       </c>
-      <c r="BM47" s="9">
-        <v>0</v>
-      </c>
-      <c r="BN47" s="9">
-        <v>0</v>
-      </c>
-      <c r="BO47" s="9">
+      <c r="BM47">
+        <v>0</v>
+      </c>
+      <c r="BN47">
+        <v>0</v>
+      </c>
+      <c r="BO47">
         <v>3.9048215282013299E-2</v>
       </c>
-      <c r="BP47" s="9">
+      <c r="BP47">
         <v>0</v>
       </c>
       <c r="BW47" t="s">
@@ -3475,8 +3626,11 @@
       <c r="BX47">
         <v>15</v>
       </c>
-    </row>
-    <row r="48" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="BY47" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="48" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -3534,22 +3688,22 @@
       <c r="BJ48">
         <v>16</v>
       </c>
-      <c r="BK48" s="9">
+      <c r="BK48">
         <v>0.27976033425320701</v>
       </c>
-      <c r="BL48" s="9">
+      <c r="BL48">
         <v>0.21102217392657599</v>
       </c>
-      <c r="BM48" s="9">
+      <c r="BM48">
         <v>0.73824332706682805</v>
       </c>
-      <c r="BN48" s="9">
+      <c r="BN48">
         <v>0.27976033425320701</v>
       </c>
-      <c r="BO48" s="9">
+      <c r="BO48">
         <v>0.221964769038522</v>
       </c>
-      <c r="BP48" s="9">
+      <c r="BP48">
         <v>0.26961343445188801</v>
       </c>
       <c r="BW48" t="s">
@@ -3558,8 +3712,11 @@
       <c r="BX48">
         <v>16</v>
       </c>
-    </row>
-    <row r="49" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -3617,22 +3774,22 @@
       <c r="BJ49">
         <v>17</v>
       </c>
-      <c r="BK49" s="9">
+      <c r="BK49">
         <v>0.46949907797243401</v>
       </c>
-      <c r="BL49" s="9">
-        <v>1</v>
-      </c>
-      <c r="BM49" s="9">
+      <c r="BL49">
+        <v>1</v>
+      </c>
+      <c r="BM49">
         <v>0.17311064529102299</v>
       </c>
-      <c r="BN49" s="9">
+      <c r="BN49">
         <v>0.46949907797243401</v>
       </c>
-      <c r="BO49" s="9">
+      <c r="BO49">
         <v>0.56949907797243404</v>
       </c>
-      <c r="BP49" s="9">
+      <c r="BP49">
         <v>0.50412120703063801</v>
       </c>
       <c r="BW49" t="s">
@@ -3641,8 +3798,11 @@
       <c r="BX49">
         <v>17</v>
       </c>
-    </row>
-    <row r="50" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY49" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>17</v>
       </c>
@@ -3700,22 +3860,22 @@
       <c r="BJ50">
         <v>18</v>
       </c>
-      <c r="BK50" s="9">
+      <c r="BK50">
         <v>0.51114327604916598</v>
       </c>
-      <c r="BL50" s="9">
+      <c r="BL50">
         <v>0.67937469217648705</v>
       </c>
-      <c r="BM50" s="9">
+      <c r="BM50">
         <v>0.17619955842436399</v>
       </c>
-      <c r="BN50" s="9">
+      <c r="BN50">
         <v>0.51114327604916598</v>
       </c>
-      <c r="BO50" s="9">
+      <c r="BO50">
         <v>0.54701821448446297</v>
       </c>
-      <c r="BP50" s="9">
+      <c r="BP50">
         <v>0.482258126169336</v>
       </c>
       <c r="BW50" t="s">
@@ -3724,8 +3884,11 @@
       <c r="BX50">
         <v>18</v>
       </c>
-    </row>
-    <row r="51" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY50" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -3783,22 +3946,22 @@
       <c r="BJ51">
         <v>19</v>
       </c>
-      <c r="BK51" s="9">
+      <c r="BK51">
         <v>0.30663855232489801</v>
       </c>
-      <c r="BL51" s="9">
+      <c r="BL51">
         <v>0.589091367411266</v>
       </c>
-      <c r="BM51" s="9">
-        <v>1</v>
-      </c>
-      <c r="BN51" s="9">
+      <c r="BM51">
+        <v>1</v>
+      </c>
+      <c r="BN51">
         <v>0.30663855232489801</v>
       </c>
-      <c r="BO51" s="9">
+      <c r="BO51">
         <v>0.32445682580715202</v>
       </c>
-      <c r="BP51" s="9">
+      <c r="BP51">
         <v>0.42445682580715199</v>
       </c>
       <c r="BW51" t="s">
@@ -3807,8 +3970,11 @@
       <c r="BX51">
         <v>19</v>
       </c>
-    </row>
-    <row r="52" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY51" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -3866,22 +4032,22 @@
       <c r="BJ52">
         <v>20</v>
       </c>
-      <c r="BK52" s="9">
+      <c r="BK52">
         <v>0.70401656549717595</v>
       </c>
-      <c r="BL52" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM52" s="9">
-        <v>0</v>
-      </c>
-      <c r="BN52" s="9">
+      <c r="BL52">
+        <v>0</v>
+      </c>
+      <c r="BM52">
+        <v>0</v>
+      </c>
+      <c r="BN52">
         <v>0.70401656549717595</v>
       </c>
-      <c r="BO52" s="9">
+      <c r="BO52">
         <v>0.60401656549717597</v>
       </c>
-      <c r="BP52" s="9">
+      <c r="BP52">
         <v>0.50401656549717599</v>
       </c>
       <c r="BW52" t="s">
@@ -3890,8 +4056,11 @@
       <c r="BX52">
         <v>20</v>
       </c>
-    </row>
-    <row r="53" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY52" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3949,22 +4118,22 @@
       <c r="BJ53">
         <v>21</v>
       </c>
-      <c r="BK53" s="9">
+      <c r="BK53">
         <v>0.34719607743012598</v>
       </c>
-      <c r="BL53" s="9">
-        <v>0</v>
-      </c>
-      <c r="BM53" s="9">
+      <c r="BL53">
+        <v>0</v>
+      </c>
+      <c r="BM53">
         <v>0.85749105466910802</v>
       </c>
-      <c r="BN53" s="9">
+      <c r="BN53">
         <v>0.34719607743012598</v>
       </c>
-      <c r="BO53" s="9">
+      <c r="BO53">
         <v>0.247196077430126</v>
       </c>
-      <c r="BP53" s="9">
+      <c r="BP53">
         <v>0.31869428836394698</v>
       </c>
       <c r="BW53" t="s">
@@ -3973,8 +4142,11 @@
       <c r="BX53">
         <v>21</v>
       </c>
-    </row>
-    <row r="54" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BY53" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK54" t="s">
         <v>55</v>
       </c>
@@ -3984,8 +4156,17 @@
       <c r="AM54" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="55" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW54" t="s">
+        <v>55</v>
+      </c>
+      <c r="BX54">
+        <v>22</v>
+      </c>
+      <c r="BY54" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="55" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK55" t="s">
         <v>54</v>
       </c>
@@ -3995,8 +4176,17 @@
       <c r="AM55" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="56" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW55" t="s">
+        <v>54</v>
+      </c>
+      <c r="BX55">
+        <v>23</v>
+      </c>
+      <c r="BY55" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="56" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK56" t="s">
         <v>53</v>
       </c>
@@ -4006,8 +4196,17 @@
       <c r="AM56" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="57" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW56" t="s">
+        <v>53</v>
+      </c>
+      <c r="BX56">
+        <v>24</v>
+      </c>
+      <c r="BY56" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK57" t="s">
         <v>52</v>
       </c>
@@ -4025,8 +4224,17 @@
       <c r="AS57" s="1"/>
       <c r="AT57" s="1"/>
       <c r="AU57" s="1"/>
-    </row>
-    <row r="58" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW57" t="s">
+        <v>52</v>
+      </c>
+      <c r="BX57">
+        <v>25</v>
+      </c>
+      <c r="BY57" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="58" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK58" t="s">
         <v>60</v>
       </c>
@@ -4044,8 +4252,17 @@
       <c r="AS58" s="1"/>
       <c r="AT58" s="1"/>
       <c r="AU58" s="1"/>
-    </row>
-    <row r="59" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW58" t="s">
+        <v>60</v>
+      </c>
+      <c r="BX58">
+        <v>26</v>
+      </c>
+      <c r="BY58" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK59" t="s">
         <v>51</v>
       </c>
@@ -4055,8 +4272,17 @@
       <c r="AM59" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="60" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW59" t="s">
+        <v>51</v>
+      </c>
+      <c r="BX59">
+        <v>27</v>
+      </c>
+      <c r="BY59" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60" spans="1:81" x14ac:dyDescent="0.25">
       <c r="AK60" t="s">
         <v>50</v>
       </c>
@@ -4066,219 +4292,207 @@
       <c r="AM60" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="63" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="BW60" t="s">
+        <v>50</v>
+      </c>
+      <c r="BX60">
+        <v>28</v>
+      </c>
+      <c r="BY60" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="63" spans="1:81" x14ac:dyDescent="0.25">
       <c r="Z63" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="64" spans="1:88" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="64" spans="1:81" x14ac:dyDescent="0.25">
       <c r="Z64" t="str" cm="1">
-        <f t="array" ref="Z64:CJ64">_xlfn.TEXTSPLIT(Z63,",")</f>
-        <v>0.5018309634301501</v>
+        <f t="array" ref="Z64:CC64">_xlfn.TEXTSPLIT(Z63,",")</f>
+        <v>0.4489769376909381</v>
       </c>
       <c r="AA64" t="str">
-        <v xml:space="preserve"> 0.7423451363740952</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AB64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AC64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.2200813583097922</v>
       </c>
       <c r="AD64" t="str">
-        <v xml:space="preserve"> 0.7889671898460878</v>
+        <v xml:space="preserve"> 0.36904127870754105</v>
       </c>
       <c r="AE64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.5734997567308384</v>
       </c>
       <c r="AF64" t="str">
-        <v xml:space="preserve"> 0.5801904002480903</v>
+        <v xml:space="preserve"> 0.7609641739977115</v>
       </c>
       <c r="AG64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AH64" t="str">
-        <v xml:space="preserve"> 0.26450840963181244</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AI64" t="str">
-        <v xml:space="preserve"> 0.49188495725867865</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AJ64" t="str">
-        <v xml:space="preserve"> 0.4170883075336374</v>
+        <v xml:space="preserve"> 0.8855302018224294</v>
       </c>
       <c r="AK64" t="str">
-        <v xml:space="preserve"> 0.09983441078009811</v>
+        <v xml:space="preserve"> 0.8306653004086676</v>
       </c>
       <c r="AL64" t="str">
-        <v xml:space="preserve"> 0.3125999621707864</v>
+        <v xml:space="preserve"> 0.5377170358339709</v>
       </c>
       <c r="AM64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.6550543815442608</v>
       </c>
       <c r="AN64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.2772477549959537</v>
       </c>
       <c r="AO64" t="str">
-        <v xml:space="preserve"> 0.27976033425320757</v>
+        <v xml:space="preserve"> 0.9592308396183514</v>
       </c>
       <c r="AP64" t="str">
-        <v xml:space="preserve"> 0.469499077972434</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AQ64" t="str">
-        <v xml:space="preserve"> 0.5111432760491664</v>
+        <v xml:space="preserve"> 0.24293859078887203</v>
       </c>
       <c r="AR64" t="str">
-        <v xml:space="preserve"> 0.30663855232489895</v>
+        <v xml:space="preserve"> 0.2529414637771258</v>
       </c>
       <c r="AS64" t="str">
-        <v xml:space="preserve"> 0.7040165654971762</v>
+        <v xml:space="preserve"> 0.9405997864481604</v>
       </c>
       <c r="AT64" t="str">
-        <v xml:space="preserve"> 0.3471960774301261</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AU64" t="str">
-        <v xml:space="preserve"> 0.47628480507854354</v>
+        <v xml:space="preserve"> 0.8282849886177859</v>
       </c>
       <c r="AV64" t="str">
-        <v xml:space="preserve"> 0.8423451363740951</v>
+        <v xml:space="preserve"> 0.7886381793044395</v>
       </c>
       <c r="AW64" t="str">
-        <v xml:space="preserve"> 0.014705895432485551</v>
+        <v xml:space="preserve"> 0.24788606446216535</v>
       </c>
       <c r="AX64" t="str">
-        <v xml:space="preserve"> 0.9956599374568458</v>
+        <v xml:space="preserve"> 0.4452603904961968</v>
       </c>
       <c r="AY64" t="str">
-        <v xml:space="preserve"> 0.7078432854533878</v>
+        <v xml:space="preserve"> 0.8513638103721802</v>
       </c>
       <c r="AZ64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.09766786771815637</v>
       </c>
       <c r="BA64" t="str">
-        <v xml:space="preserve"> 0.48019040024809034</v>
+        <v xml:space="preserve"> 0.4317827066736215</v>
       </c>
       <c r="BB64" t="str">
-        <v xml:space="preserve"> 0.013677038307942603</v>
+        <v xml:space="preserve"> 0.38365795363489325</v>
       </c>
       <c r="BC64" t="str">
-        <v xml:space="preserve"> 0.16450840963181243</v>
+        <v xml:space="preserve"> 0.4474496490628219</v>
       </c>
       <c r="BD64" t="str">
-        <v xml:space="preserve"> 0.4623716489913056</v>
+        <v xml:space="preserve"> 0.8204377341428768</v>
       </c>
       <c r="BE64" t="str">
-        <v xml:space="preserve"> 0.31708830753363737</v>
+        <v xml:space="preserve"> 0.17300304887729573</v>
       </c>
       <c r="BF64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.33618881620573426</v>
       </c>
       <c r="BG64" t="str">
-        <v xml:space="preserve"> 0.34874940380617453</v>
+        <v xml:space="preserve"> 0.07601503063487242</v>
       </c>
       <c r="BH64" t="str">
-        <v xml:space="preserve"> 0.9</v>
+        <v xml:space="preserve"> 0.09118924302373758</v>
       </c>
       <c r="BI64" t="str">
-        <v xml:space="preserve"> 0.03904821528201339</v>
+        <v xml:space="preserve"> 0.5503333105413887</v>
       </c>
       <c r="BJ64" t="str">
-        <v xml:space="preserve"> 0.22196476903852289</v>
+        <v xml:space="preserve"> 1.317969980390527</v>
       </c>
       <c r="BK64" t="str">
-        <v xml:space="preserve"> 0.569499077972434</v>
+        <v xml:space="preserve"> 0.6145414649828274</v>
       </c>
       <c r="BL64" t="str">
-        <v xml:space="preserve"> 0.5470182144844639</v>
+        <v xml:space="preserve"> 0.3519713726795352</v>
       </c>
       <c r="BM64" t="str">
-        <v xml:space="preserve"> 0.32445682580715235</v>
+        <v xml:space="preserve"> 0.2963622514040038</v>
       </c>
       <c r="BN64" t="str">
-        <v xml:space="preserve"> 0.6040165654971762</v>
+        <v xml:space="preserve"> 0.276955383826611</v>
       </c>
       <c r="BO64" t="str">
-        <v xml:space="preserve"> 0.2471960774301261</v>
+        <v xml:space="preserve"> 0.8005728430930316</v>
       </c>
       <c r="BP64" t="str">
-        <v xml:space="preserve"> 0.5728993986822584</v>
+        <v xml:space="preserve"> 0.02427733053940036</v>
       </c>
       <c r="BQ64" t="str">
-        <v xml:space="preserve"> 0.9423451363740951</v>
+        <v xml:space="preserve"> 1.6067053727056138</v>
       </c>
       <c r="BR64" t="str">
-        <v xml:space="preserve"> 0.08947250274492421</v>
+        <v xml:space="preserve"> 0.4862103185448709</v>
       </c>
       <c r="BS64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.10861069729595417</v>
       </c>
       <c r="BT64" t="str">
-        <v xml:space="preserve"> 0.6466465957242477</v>
+        <v xml:space="preserve"> 0.29557917692469254</v>
       </c>
       <c r="BU64" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.8715150786731626</v>
       </c>
       <c r="BV64" t="str">
-        <v xml:space="preserve"> 0.5074274005848062</v>
+        <v xml:space="preserve"> 0.839398210617237</v>
       </c>
       <c r="BW64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.6870816863298209</v>
       </c>
       <c r="BX64" t="str">
-        <v xml:space="preserve"> 0.14289177800553857</v>
+        <v xml:space="preserve"> 0.6557872328730052</v>
       </c>
       <c r="BY64" t="str">
-        <v xml:space="preserve"> 0.5623716489913057</v>
+        <v xml:space="preserve"> 0.13697399763482626</v>
       </c>
       <c r="BZ64" t="str">
-        <v xml:space="preserve"> 0.24690025994053244</v>
+        <v xml:space="preserve"> 0.16569205613001692</v>
       </c>
       <c r="CA64" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.7745538427122949</v>
       </c>
       <c r="CB64" t="str">
-        <v xml:space="preserve"> 0.30105336034734864</v>
+        <v xml:space="preserve"> 0.2968141695339541</v>
       </c>
       <c r="CC64" t="str">
-        <v xml:space="preserve"> 0.9065068994520135</v>
-      </c>
-      <c r="CD64" t="str">
-        <v xml:space="preserve"> 0.0</v>
-      </c>
-      <c r="CE64" t="str">
-        <v xml:space="preserve"> 0.26961343445188857</v>
-      </c>
-      <c r="CF64" t="str">
-        <v xml:space="preserve"> 0.5041212070306388</v>
-      </c>
-      <c r="CG64" t="str">
-        <v xml:space="preserve"> 0.48225812616933666</v>
-      </c>
-      <c r="CH64" t="str">
-        <v xml:space="preserve"> 0.4244568258071524</v>
-      </c>
-      <c r="CI64" t="str">
-        <v xml:space="preserve"> 0.5040165654971762</v>
-      </c>
-      <c r="CJ64" t="str">
-        <v xml:space="preserve"> 0.31869428836394775</v>
-      </c>
-    </row>
-    <row r="65" spans="25:56" x14ac:dyDescent="0.25">
+        <v xml:space="preserve"> 1.5314411976433369</v>
+      </c>
+    </row>
+    <row r="65" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y65">
         <v>1</v>
       </c>
       <c r="Z65" s="3" t="str" cm="1">
-        <f t="array" ref="Z65:Z127">TRANSPOSE(_xlfn.ANCHORARRAY(Z64))</f>
-        <v>0.5018309634301501</v>
-      </c>
-    </row>
-    <row r="66" spans="25:56" x14ac:dyDescent="0.25">
+        <f t="array" ref="Z65:Z120">TRANSPOSE(_xlfn.ANCHORARRAY(Z64))</f>
+        <v>0.4489769376909381</v>
+      </c>
+    </row>
+    <row r="66" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y66">
         <v>2</v>
       </c>
       <c r="Z66" s="2" t="str">
-        <v xml:space="preserve"> 0.7423451363740952</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AZ66" s="3">
         <v>0.33831719711374802</v>
@@ -4298,13 +4512,17 @@
         <f>SUM(_xlfn.ANCHORARRAY(BC66))</f>
         <v>7.9290406405481404</v>
       </c>
-    </row>
-    <row r="67" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH66" t="str">
+        <f>_xlfn.TEXTJOIN("#",TRUE,BH68:BH88)</f>
+        <v>0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126#0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0#0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108#0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126#0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0#0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108</v>
+      </c>
+    </row>
+    <row r="67" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y67">
         <v>3</v>
       </c>
       <c r="Z67" s="3" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AZ67" s="2">
         <v>0.93466713178917704</v>
@@ -4313,23 +4531,27 @@
         <v>34</v>
       </c>
       <c r="BB67">
-        <f t="shared" ref="BB67:BB86" si="0">AZ67-BA67</f>
+        <f t="shared" ref="BB67:BB86" si="1">AZ67-BA67</f>
         <v>-6.5332868210822959E-2</v>
       </c>
       <c r="BC67">
         <v>6.5332868210822959E-2</v>
       </c>
-    </row>
-    <row r="68" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH67" t="str">
+        <f>_xlfn.REGEXREPLACE(BH66," ","")</f>
+        <v>0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126#0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0#0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108#0.50183096343015#0.742345136374095#0#1#0.788967189846087#1#0.58019040024809#0#0.264508409631812#0.491884957258678#0.417088307533637#0.0998344107800981#0.312599962170786#1#0#0.279760334253207#0.469499077972434#0.511143276049166#0.306638552324898#0.704016565497176#0.347196077430126#0.372269208241967#1#0.573529477162427#0.478299687284229#0.0943804780364997#1#0#0.568385191539713#0#0.352433458663134#0#0#0.68074720817694#0#0.695241076410066#0.211022173926576#1#0.679374692176487#0.589091367411266#0#0#0.983072968018574#1#0.873833036562193#0.577481377245474#0.194016551354299#1#0.636185001683579#0#0.39191684186863#1#0.149059762034475#0#0.26151978270587#0.532534497260067#0#0.738243327066828#0.173110645291023#0.176199558424364#1#0#0.857491054669108</v>
+      </c>
+    </row>
+    <row r="68" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y68">
         <v>4</v>
       </c>
       <c r="Z68" s="2" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.2200813583097922</v>
       </c>
       <c r="AB68" t="str">
         <f>_xlfn.TEXTJOIN("#",FALSE,Z86:Z92)</f>
-        <v xml:space="preserve"> 0.47628480507854354# 0.8423451363740951# 0.014705895432485551# 0.9956599374568458# 0.7078432854533878# 1.0# 0.48019040024809034</v>
+        <v xml:space="preserve"> 0.8282849886177859# 0.7886381793044395# 0.24788606446216535# 0.4452603904961968# 0.8513638103721802# 0.09766786771815637# 0.4317827066736215</v>
       </c>
       <c r="AZ68" s="3">
         <v>9.3176192652155904E-2</v>
@@ -4338,19 +4560,22 @@
         <v>35</v>
       </c>
       <c r="BB68">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.3176192652155904E-2</v>
       </c>
       <c r="BC68">
         <v>9.3176192652155904E-2</v>
       </c>
-    </row>
-    <row r="69" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH68" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y69">
         <v>5</v>
       </c>
       <c r="Z69" s="3" t="str">
-        <v xml:space="preserve"> 0.7889671898460878</v>
+        <v xml:space="preserve"> 0.36904127870754105</v>
       </c>
       <c r="AZ69" s="2">
         <v>0</v>
@@ -4359,19 +4584,22 @@
         <v>35</v>
       </c>
       <c r="BB69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BC69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH69" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="70" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y70">
         <v>6</v>
       </c>
       <c r="Z70" s="2" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.5734997567308384</v>
       </c>
       <c r="AB70" t="s">
         <v>56</v>
@@ -4383,19 +4611,22 @@
         <v>34</v>
       </c>
       <c r="BB70">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.24890097536999201</v>
       </c>
       <c r="BC70">
         <v>0.24890097536999201</v>
       </c>
-    </row>
-    <row r="71" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH70" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="71" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y71">
         <v>7</v>
       </c>
       <c r="Z71" s="3" t="str">
-        <v xml:space="preserve"> 0.5801904002480903</v>
+        <v xml:space="preserve"> 0.7609641739977115</v>
       </c>
       <c r="AB71" t="str">
         <f>_xlfn.REGEXREPLACE(AB70," ",,)</f>
@@ -4408,19 +4639,19 @@
         <v>34</v>
       </c>
       <c r="BB71">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BC71">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="72" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y72">
         <v>8</v>
       </c>
       <c r="Z72" s="2" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AB72" t="s">
         <v>57</v>
@@ -4432,19 +4663,19 @@
         <v>34</v>
       </c>
       <c r="BB72">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-3.8152113662125009E-2</v>
       </c>
       <c r="BC72">
         <v>3.8152113662125009E-2</v>
       </c>
     </row>
-    <row r="73" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="73" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y73">
         <v>9</v>
       </c>
       <c r="Z73" s="3" t="str">
-        <v xml:space="preserve"> 0.26450840963181244</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AZ73" s="2">
         <v>0</v>
@@ -4453,19 +4684,22 @@
         <v>35</v>
       </c>
       <c r="BB73">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BC73">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="25:56" x14ac:dyDescent="0.25">
+      <c r="BH73" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="74" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y74">
         <v>10</v>
       </c>
       <c r="Z74" s="2" t="str">
-        <v xml:space="preserve"> 0.49188495725867865</v>
+        <v xml:space="preserve"> 1</v>
       </c>
       <c r="AZ74" s="3">
         <v>1</v>
@@ -4474,19 +4708,19 @@
         <v>36</v>
       </c>
       <c r="BB74">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13852660842636</v>
       </c>
       <c r="BC74">
         <v>0.13852660842636</v>
       </c>
     </row>
-    <row r="75" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="75" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y75">
         <v>11</v>
       </c>
       <c r="Z75" s="3" t="str">
-        <v xml:space="preserve"> 0.4170883075336374</v>
+        <v xml:space="preserve"> 0.8855302018224294</v>
       </c>
       <c r="AZ75" s="2">
         <v>0.55293794800527796</v>
@@ -4495,19 +4729,19 @@
         <v>34</v>
       </c>
       <c r="BB75">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.44706205199472204</v>
       </c>
       <c r="BC75">
         <v>0.44706205199472204</v>
       </c>
     </row>
-    <row r="76" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="76" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y76">
         <v>12</v>
       </c>
       <c r="Z76" s="2" t="str">
-        <v xml:space="preserve"> 0.09983441078009811</v>
+        <v xml:space="preserve"> 0.8306653004086676</v>
       </c>
       <c r="AZ76" s="3">
         <v>0.59671345821399002</v>
@@ -4516,19 +4750,19 @@
         <v>37</v>
       </c>
       <c r="BB76">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.3686848516020014E-2</v>
       </c>
       <c r="BC76">
         <v>5.3686848516020014E-2</v>
       </c>
     </row>
-    <row r="77" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="77" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y77">
         <v>13</v>
       </c>
       <c r="Z77" s="3" t="str">
-        <v xml:space="preserve"> 0.3125999621707864</v>
+        <v xml:space="preserve"> 0.5377170358339709</v>
       </c>
       <c r="AZ77" s="2">
         <v>0</v>
@@ -4537,19 +4771,19 @@
         <v>34</v>
       </c>
       <c r="BB77">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="BC77">
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="78" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y78">
         <v>14</v>
       </c>
       <c r="Z78" s="2" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.6550543815442608</v>
       </c>
       <c r="AZ78" s="3">
         <v>1</v>
@@ -4558,19 +4792,19 @@
         <v>35</v>
       </c>
       <c r="BB78">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="BC78">
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="79" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y79">
         <v>15</v>
       </c>
       <c r="Z79" s="3" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.2772477549959537</v>
       </c>
       <c r="AZ79" s="2">
         <v>0</v>
@@ -4579,19 +4813,19 @@
         <v>38</v>
       </c>
       <c r="BB79">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.17621606443353</v>
       </c>
       <c r="BC79">
         <v>0.17621606443353</v>
       </c>
     </row>
-    <row r="80" spans="25:56" x14ac:dyDescent="0.25">
+    <row r="80" spans="25:60" x14ac:dyDescent="0.25">
       <c r="Y80">
         <v>16</v>
       </c>
       <c r="Z80" s="2" t="str">
-        <v xml:space="preserve"> 0.27976033425320757</v>
+        <v xml:space="preserve"> 0.9592308396183514</v>
       </c>
       <c r="AZ80" s="3">
         <v>0</v>
@@ -4600,7 +4834,7 @@
         <v>34</v>
       </c>
       <c r="BB80">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="BC80">
@@ -4612,7 +4846,7 @@
         <v>17</v>
       </c>
       <c r="Z81" s="3" t="str">
-        <v xml:space="preserve"> 0.469499077972434</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AZ81" s="2">
         <v>1</v>
@@ -4621,7 +4855,7 @@
         <v>39</v>
       </c>
       <c r="BB81">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.58957907790050801</v>
       </c>
       <c r="BC81">
@@ -4633,7 +4867,7 @@
         <v>18</v>
       </c>
       <c r="Z82" s="2" t="str">
-        <v xml:space="preserve"> 0.5111432760491664</v>
+        <v xml:space="preserve"> 0.24293859078887203</v>
       </c>
       <c r="AZ82" s="3">
         <v>0</v>
@@ -4642,7 +4876,7 @@
         <v>40</v>
       </c>
       <c r="BB82">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.93748321022143899</v>
       </c>
       <c r="BC82">
@@ -4654,7 +4888,7 @@
         <v>19</v>
       </c>
       <c r="Z83" s="3" t="str">
-        <v xml:space="preserve"> 0.30663855232489895</v>
+        <v xml:space="preserve"> 0.2529414637771258</v>
       </c>
       <c r="AZ83" s="2">
         <v>2.1401265694797498E-3</v>
@@ -4663,7 +4897,7 @@
         <v>34</v>
       </c>
       <c r="BB83">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.99785987343052029</v>
       </c>
       <c r="BC83">
@@ -4675,7 +4909,7 @@
         <v>20</v>
       </c>
       <c r="Z84" s="2" t="str">
-        <v xml:space="preserve"> 0.7040165654971762</v>
+        <v xml:space="preserve"> 0.9405997864481604</v>
       </c>
       <c r="AZ84" s="3">
         <v>0.37166843346534201</v>
@@ -4684,7 +4918,7 @@
         <v>41</v>
       </c>
       <c r="BB84">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.8902838744676018E-2</v>
       </c>
       <c r="BC84">
@@ -4696,7 +4930,7 @@
         <v>21</v>
       </c>
       <c r="Z85" s="3" t="str">
-        <v xml:space="preserve"> 0.3471960774301261</v>
+        <v xml:space="preserve"> 0</v>
       </c>
       <c r="AZ85" s="2">
         <v>0.16946907320228299</v>
@@ -4705,7 +4939,7 @@
         <v>42</v>
       </c>
       <c r="BB85">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.15121010424644088</v>
       </c>
       <c r="BC85">
@@ -4717,7 +4951,7 @@
         <v>22</v>
       </c>
       <c r="Z86" s="2" t="str">
-        <v xml:space="preserve"> 0.47628480507854354</v>
+        <v xml:space="preserve"> 0.8282849886177859</v>
       </c>
       <c r="AZ86" s="3">
         <v>0</v>
@@ -4726,7 +4960,7 @@
         <v>43</v>
       </c>
       <c r="BB86">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.28901297450699598</v>
       </c>
       <c r="BC86">
@@ -4738,7 +4972,7 @@
         <v>23</v>
       </c>
       <c r="Z87" s="3" t="str">
-        <v xml:space="preserve"> 0.8423451363740951</v>
+        <v xml:space="preserve"> 0.7886381793044395</v>
       </c>
       <c r="BA87" t="s">
         <v>44</v>
@@ -4749,7 +4983,7 @@
         <v>24</v>
       </c>
       <c r="Z88" s="2" t="str">
-        <v xml:space="preserve"> 0.014705895432485551</v>
+        <v xml:space="preserve"> 0.24788606446216535</v>
       </c>
       <c r="AI88" t="s">
         <v>58</v>
@@ -4763,7 +4997,7 @@
         <v>25</v>
       </c>
       <c r="Z89" s="3" t="str">
-        <v xml:space="preserve"> 0.9956599374568458</v>
+        <v xml:space="preserve"> 0.4452603904961968</v>
       </c>
       <c r="AH89" t="s">
         <v>58</v>
@@ -4783,7 +5017,7 @@
         <v>26</v>
       </c>
       <c r="Z90" s="2" t="str">
-        <v xml:space="preserve"> 0.7078432854533878</v>
+        <v xml:space="preserve"> 0.8513638103721802</v>
       </c>
       <c r="AH90">
         <v>1</v>
@@ -4809,7 +5043,7 @@
         <v>27</v>
       </c>
       <c r="Z91" s="3" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.09766786771815637</v>
       </c>
       <c r="AG91">
         <v>1</v>
@@ -4819,19 +5053,19 @@
       </c>
       <c r="AI91" s="5">
         <f ca="1">RAND()*0.1-0.05</f>
-        <v>-3.3845043940489053E-2</v>
+        <v>7.4222227538069258E-3</v>
       </c>
       <c r="AJ91" s="5">
         <f ca="1">MIN(MAX(AH91+AI91,0),1)</f>
-        <v>0</v>
+        <v>7.4222227538069258E-3</v>
       </c>
       <c r="AK91" s="5">
-        <f t="shared" ref="AK91:AK111" ca="1" si="1">RAND()*0.1-0.05</f>
-        <v>7.6510679195523554E-3</v>
+        <f t="shared" ref="AK91:AK111" ca="1" si="2">RAND()*0.1-0.05</f>
+        <v>1.5080864872341754E-3</v>
       </c>
       <c r="AL91" s="5">
         <f ca="1">MIN(MAX(AJ91+AK91,0),1)</f>
-        <v>7.6510679195523554E-3</v>
+        <v>8.9303092410411011E-3</v>
       </c>
       <c r="BA91" t="s">
         <v>47</v>
@@ -4842,7 +5076,7 @@
         <v>28</v>
       </c>
       <c r="Z92" s="2" t="str">
-        <v xml:space="preserve"> 0.48019040024809034</v>
+        <v xml:space="preserve"> 0.4317827066736215</v>
       </c>
       <c r="AG92">
         <v>2</v>
@@ -4851,20 +5085,20 @@
         <v>0.838073450710207</v>
       </c>
       <c r="AI92" s="5">
-        <f t="shared" ref="AI92:AI111" ca="1" si="2">RAND()*0.1-0.05</f>
-        <v>-4.9364111418032965E-2</v>
+        <f t="shared" ref="AI92:AI111" ca="1" si="3">RAND()*0.1-0.05</f>
+        <v>-4.4943789075088669E-3</v>
       </c>
       <c r="AJ92" s="5">
-        <f t="shared" ref="AJ92:AJ111" ca="1" si="3">MIN(MAX(AH92+AI92,0),1)</f>
-        <v>0.78870933929217402</v>
+        <f t="shared" ref="AJ92:AJ111" ca="1" si="4">MIN(MAX(AH92+AI92,0),1)</f>
+        <v>0.83357907180269808</v>
       </c>
       <c r="AK92" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-4.5141789742012578E-2</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>-2.1309478454764854E-2</v>
       </c>
       <c r="AL92" s="5">
-        <f t="shared" ref="AL92:AL111" ca="1" si="4">MIN(MAX(AJ92+AK92,0),1)</f>
-        <v>0.74356754955016147</v>
+        <f t="shared" ref="AL92:AL111" ca="1" si="5">MIN(MAX(AJ92+AK92,0),1)</f>
+        <v>0.81226959334793325</v>
       </c>
       <c r="BA92" t="s">
         <v>48</v>
@@ -4875,7 +5109,7 @@
         <v>29</v>
       </c>
       <c r="Z93" t="str">
-        <v xml:space="preserve"> 0.013677038307942603</v>
+        <v xml:space="preserve"> 0.38365795363489325</v>
       </c>
       <c r="AG93">
         <v>3</v>
@@ -4884,20 +5118,20 @@
         <v>0.36941805210713202</v>
       </c>
       <c r="AI93" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-4.4191793955125513E-2</v>
+      </c>
+      <c r="AJ93" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.32522625815200651</v>
+      </c>
+      <c r="AK93" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-5.6464485745091886E-3</v>
-      </c>
-      <c r="AJ93" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.36377160353262283</v>
-      </c>
-      <c r="AK93" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-4.5673298263072509E-2</v>
+        <v>-3.055772513343763E-2</v>
       </c>
       <c r="AL93" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.3180983052695503</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.29466853301856888</v>
       </c>
       <c r="BA93" t="s">
         <v>34</v>
@@ -4908,7 +5142,7 @@
         <v>30</v>
       </c>
       <c r="Z94" t="str">
-        <v xml:space="preserve"> 0.16450840963181243</v>
+        <v xml:space="preserve"> 0.4474496490628219</v>
       </c>
       <c r="AG94">
         <v>4</v>
@@ -4917,20 +5151,20 @@
         <v>0.772175920311859</v>
       </c>
       <c r="AI94" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-4.2316829345673768E-2</v>
+      </c>
+      <c r="AJ94" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.72985909096618529</v>
+      </c>
+      <c r="AK94" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-3.581690137964743E-2</v>
-      </c>
-      <c r="AJ94" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.73635901893221156</v>
-      </c>
-      <c r="AK94" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-4.2556740711018594E-2</v>
+        <v>-7.072134185295044E-3</v>
       </c>
       <c r="AL94" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.693802278221193</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.72278695678089022</v>
       </c>
     </row>
     <row r="95" spans="25:55" x14ac:dyDescent="0.25">
@@ -4938,7 +5172,7 @@
         <v>31</v>
       </c>
       <c r="Z95" t="str">
-        <v xml:space="preserve"> 0.4623716489913056</v>
+        <v xml:space="preserve"> 0.8204377341428768</v>
       </c>
       <c r="AG95">
         <v>5</v>
@@ -4947,20 +5181,20 @@
         <v>0.61234593074099897</v>
       </c>
       <c r="AI95" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-3.8784985724824889E-2</v>
+      </c>
+      <c r="AJ95" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.57356094501617405</v>
+      </c>
+      <c r="AK95" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-4.2076205457542516E-2</v>
-      </c>
-      <c r="AJ95" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.57026972528345643</v>
-      </c>
-      <c r="AK95" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-1.73678674872376E-2</v>
+        <v>-4.0066846839539962E-2</v>
       </c>
       <c r="AL95" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.55290185779621881</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.53349409817663407</v>
       </c>
     </row>
     <row r="96" spans="25:55" x14ac:dyDescent="0.25">
@@ -4968,7 +5202,7 @@
         <v>32</v>
       </c>
       <c r="Z96" t="str">
-        <v xml:space="preserve"> 0.31708830753363737</v>
+        <v xml:space="preserve"> 0.17300304887729573</v>
       </c>
       <c r="AG96">
         <v>6</v>
@@ -4977,20 +5211,20 @@
         <v>0</v>
       </c>
       <c r="AI96" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>4.6298989919132227E-2</v>
+      </c>
+      <c r="AJ96" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>4.6298989919132227E-2</v>
+      </c>
+      <c r="AK96" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-3.3891669187567794E-2</v>
-      </c>
-      <c r="AJ96" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AK96" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>7.2163328842814178E-5</v>
+        <v>4.3887380250421049E-2</v>
       </c>
       <c r="AL96" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>7.2163328842814178E-5</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>9.0186370169553276E-2</v>
       </c>
     </row>
     <row r="97" spans="25:38" x14ac:dyDescent="0.25">
@@ -4998,7 +5232,7 @@
         <v>33</v>
       </c>
       <c r="Z97" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.33618881620573426</v>
       </c>
       <c r="AG97">
         <v>7</v>
@@ -5007,20 +5241,20 @@
         <v>1</v>
       </c>
       <c r="AI97" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-3.6187487179181466E-2</v>
+      </c>
+      <c r="AJ97" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.96381251282081859</v>
+      </c>
+      <c r="AK97" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-3.298501735634933E-2</v>
-      </c>
-      <c r="AJ97" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.96701498264365071</v>
-      </c>
-      <c r="AK97" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-3.723024927100136E-2</v>
+        <v>-1.8543040583565262E-2</v>
       </c>
       <c r="AL97" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.92978473337264933</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.94526947223725333</v>
       </c>
     </row>
     <row r="98" spans="25:38" x14ac:dyDescent="0.25">
@@ -5028,7 +5262,7 @@
         <v>34</v>
       </c>
       <c r="Z98" t="str">
-        <v xml:space="preserve"> 0.34874940380617453</v>
+        <v xml:space="preserve"> 0.07601503063487242</v>
       </c>
       <c r="AG98">
         <v>8</v>
@@ -5037,20 +5271,20 @@
         <v>0.27929680791088402</v>
       </c>
       <c r="AI98" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>3.5542663383942616E-2</v>
+      </c>
+      <c r="AJ98" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.31483947129482664</v>
+      </c>
+      <c r="AK98" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>2.4971249044662067E-2</v>
-      </c>
-      <c r="AJ98" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.3042680569555461</v>
-      </c>
-      <c r="AK98" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>1.2329960234936634E-2</v>
+        <v>9.9704773813933251E-3</v>
       </c>
       <c r="AL98" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.31659801719048275</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.32480994867621998</v>
       </c>
     </row>
     <row r="99" spans="25:38" x14ac:dyDescent="0.25">
@@ -5058,7 +5292,7 @@
         <v>35</v>
       </c>
       <c r="Z99" t="str">
-        <v xml:space="preserve"> 0.9</v>
+        <v xml:space="preserve"> 0.09118924302373758</v>
       </c>
       <c r="AG99">
         <v>9</v>
@@ -5067,20 +5301,20 @@
         <v>1</v>
       </c>
       <c r="AI99" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>3.5463125862199768E-2</v>
+      </c>
+      <c r="AJ99" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AK99" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-4.9721116367350708E-2</v>
-      </c>
-      <c r="AJ99" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.95027888363264934</v>
-      </c>
-      <c r="AK99" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>4.8562209555836816E-2</v>
+        <v>3.9886866876638824E-2</v>
       </c>
       <c r="AL99" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.99884109318848613</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="25:38" x14ac:dyDescent="0.25">
@@ -5088,7 +5322,7 @@
         <v>36</v>
       </c>
       <c r="Z100" t="str">
-        <v xml:space="preserve"> 0.03904821528201339</v>
+        <v xml:space="preserve"> 0.5503333105413887</v>
       </c>
       <c r="AG100">
         <v>10</v>
@@ -5097,20 +5331,20 @@
         <v>3.9908815338230499E-2</v>
       </c>
       <c r="AI100" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-5.4471486464295477E-3</v>
+      </c>
+      <c r="AJ100" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>3.4461666691800952E-2</v>
+      </c>
+      <c r="AK100" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-3.4054899829159713E-2</v>
-      </c>
-      <c r="AJ100" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>5.8539155090707867E-3</v>
-      </c>
-      <c r="AK100" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>2.4967613221292831E-2</v>
+        <v>-8.2056832968511739E-3</v>
       </c>
       <c r="AL100" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>3.0821528730363618E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>2.6255983394949778E-2</v>
       </c>
     </row>
     <row r="101" spans="25:38" x14ac:dyDescent="0.25">
@@ -5118,7 +5352,7 @@
         <v>37</v>
       </c>
       <c r="Z101" t="str">
-        <v xml:space="preserve"> 0.22196476903852289</v>
+        <v xml:space="preserve"> 1.317969980390527</v>
       </c>
       <c r="AG101">
         <v>11</v>
@@ -5127,20 +5361,20 @@
         <v>0.93716941113188901</v>
       </c>
       <c r="AI101" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-2.9140611287146147E-2</v>
+      </c>
+      <c r="AJ101" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.90802879984474283</v>
+      </c>
+      <c r="AK101" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-9.5298657755173641E-3</v>
-      </c>
-      <c r="AJ101" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.92763954535637161</v>
-      </c>
-      <c r="AK101" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-4.4291971998650009E-2</v>
+        <v>-7.4304959569160278E-4</v>
       </c>
       <c r="AL101" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.88334757335772163</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.90728575024905123</v>
       </c>
     </row>
     <row r="102" spans="25:38" x14ac:dyDescent="0.25">
@@ -5148,7 +5382,7 @@
         <v>38</v>
       </c>
       <c r="Z102" t="str">
-        <v xml:space="preserve"> 0.569499077972434</v>
+        <v xml:space="preserve"> 0.6145414649828274</v>
       </c>
       <c r="AG102">
         <v>12</v>
@@ -5157,20 +5391,20 @@
         <v>1</v>
       </c>
       <c r="AI102" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-3.1973185271086169E-2</v>
+      </c>
+      <c r="AJ102" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.96802681472891383</v>
+      </c>
+      <c r="AK102" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-3.1594339224075979E-3</v>
-      </c>
-      <c r="AJ102" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.99684056607759242</v>
-      </c>
-      <c r="AK102" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>4.8280127855138855E-2</v>
+        <v>1.4831930414386754E-2</v>
       </c>
       <c r="AL102" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.98285874514330063</v>
       </c>
     </row>
     <row r="103" spans="25:38" x14ac:dyDescent="0.25">
@@ -5178,7 +5412,7 @@
         <v>39</v>
       </c>
       <c r="Z103" t="str">
-        <v xml:space="preserve"> 0.5470182144844639</v>
+        <v xml:space="preserve"> 0.3519713726795352</v>
       </c>
       <c r="AG103">
         <v>13</v>
@@ -5187,20 +5421,20 @@
         <v>0.62226011233405598</v>
       </c>
       <c r="AI103" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>3.2816757921333858E-2</v>
+      </c>
+      <c r="AJ103" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.65507687025538985</v>
+      </c>
+      <c r="AK103" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-2.5434067624082214E-2</v>
-      </c>
-      <c r="AJ103" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.5968260447099738</v>
-      </c>
-      <c r="AK103" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-3.4715908596251857E-2</v>
+        <v>2.8497534998374568E-2</v>
       </c>
       <c r="AL103" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.56211013611372196</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.68357440525376445</v>
       </c>
     </row>
     <row r="104" spans="25:38" x14ac:dyDescent="0.25">
@@ -5208,7 +5442,7 @@
         <v>40</v>
       </c>
       <c r="Z104" t="str">
-        <v xml:space="preserve"> 0.32445682580715235</v>
+        <v xml:space="preserve"> 0.2963622514040038</v>
       </c>
       <c r="AG104">
         <v>14</v>
@@ -5217,20 +5451,20 @@
         <v>0</v>
       </c>
       <c r="AI104" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>1.8423706702841075E-2</v>
+      </c>
+      <c r="AJ104" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>1.8423706702841075E-2</v>
+      </c>
+      <c r="AK104" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>4.261825993568838E-2</v>
-      </c>
-      <c r="AJ104" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>4.261825993568838E-2</v>
-      </c>
-      <c r="AK104" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-2.850687088272974E-2</v>
+        <v>-2.1873714419607095E-2</v>
       </c>
       <c r="AL104" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>1.4111389052958639E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="25:38" x14ac:dyDescent="0.25">
@@ -5238,7 +5472,7 @@
         <v>41</v>
       </c>
       <c r="Z105" t="str">
-        <v xml:space="preserve"> 0.6040165654971762</v>
+        <v xml:space="preserve"> 0.276955383826611</v>
       </c>
       <c r="AG105">
         <v>15</v>
@@ -5247,20 +5481,20 @@
         <v>0.55344351954543602</v>
       </c>
       <c r="AI105" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-1.2918037755893855E-3</v>
+      </c>
+      <c r="AJ105" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.55215171576984667</v>
+      </c>
+      <c r="AK105" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>3.255961576973776E-3</v>
-      </c>
-      <c r="AJ105" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.55669948112240975</v>
-      </c>
-      <c r="AK105" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>3.7801770888661171E-2</v>
+        <v>-1.4717235914235148E-2</v>
       </c>
       <c r="AL105" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.59450125201107096</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.53743447985561155</v>
       </c>
     </row>
     <row r="106" spans="25:38" x14ac:dyDescent="0.25">
@@ -5268,7 +5502,7 @@
         <v>42</v>
       </c>
       <c r="Z106" t="str">
-        <v xml:space="preserve"> 0.2471960774301261</v>
+        <v xml:space="preserve"> 0.8005728430930316</v>
       </c>
       <c r="AG106">
         <v>16</v>
@@ -5277,20 +5511,20 @@
         <v>0.78854921023547897</v>
       </c>
       <c r="AI106" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>1.5964161350200803E-2</v>
+      </c>
+      <c r="AJ106" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.80451337158567982</v>
+      </c>
+      <c r="AK106" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>2.428491438785621E-2</v>
-      </c>
-      <c r="AJ106" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.81283412462333515</v>
-      </c>
-      <c r="AK106" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-3.6667352838671244E-2</v>
+        <v>-3.3166995136685792E-2</v>
       </c>
       <c r="AL106" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.77616677178466387</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.77134637644899406</v>
       </c>
     </row>
     <row r="107" spans="25:38" x14ac:dyDescent="0.25">
@@ -5298,7 +5532,7 @@
         <v>43</v>
       </c>
       <c r="Z107" t="str">
-        <v xml:space="preserve"> 0.5728993986822584</v>
+        <v xml:space="preserve"> 0.02427733053940036</v>
       </c>
       <c r="AG107">
         <v>17</v>
@@ -5307,20 +5541,20 @@
         <v>0.34360099288912299</v>
       </c>
       <c r="AI107" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>1.2097300790069508E-2</v>
+      </c>
+      <c r="AJ107" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.35569829367919248</v>
+      </c>
+      <c r="AK107" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>4.2152828773575568E-2</v>
-      </c>
-      <c r="AJ107" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.38575382166269856</v>
-      </c>
-      <c r="AK107" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>1.19995820802812E-2</v>
+        <v>-4.9381270033845848E-2</v>
       </c>
       <c r="AL107" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.39775340374297974</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.30631702364534663</v>
       </c>
     </row>
     <row r="108" spans="25:38" x14ac:dyDescent="0.25">
@@ -5328,7 +5562,7 @@
         <v>44</v>
       </c>
       <c r="Z108" t="str">
-        <v xml:space="preserve"> 0.9423451363740951</v>
+        <v xml:space="preserve"> 1.6067053727056138</v>
       </c>
       <c r="AG108">
         <v>18</v>
@@ -5337,20 +5571,20 @@
         <v>0</v>
       </c>
       <c r="AI108" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>1.4159841860335018E-2</v>
+      </c>
+      <c r="AJ108" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>1.4159841860335018E-2</v>
+      </c>
+      <c r="AK108" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>4.3845616633648152E-2</v>
-      </c>
-      <c r="AJ108" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>4.3845616633648152E-2</v>
-      </c>
-      <c r="AK108" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>4.2269733961565872E-2</v>
+        <v>-8.7068085411543678E-4</v>
       </c>
       <c r="AL108" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>8.6115350595214024E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1.3289161006219581E-2</v>
       </c>
     </row>
     <row r="109" spans="25:38" x14ac:dyDescent="0.25">
@@ -5358,7 +5592,7 @@
         <v>45</v>
       </c>
       <c r="Z109" t="str">
-        <v xml:space="preserve"> 0.08947250274492421</v>
+        <v xml:space="preserve"> 0.4862103185448709</v>
       </c>
       <c r="AG109">
         <v>19</v>
@@ -5367,20 +5601,20 @@
         <v>0.34378680064676098</v>
       </c>
       <c r="AI109" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-5.8904493262448426E-3</v>
+      </c>
+      <c r="AJ109" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.33789635132051615</v>
+      </c>
+      <c r="AK109" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1.4897609668668793E-2</v>
-      </c>
-      <c r="AJ109" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.35868441031542975</v>
-      </c>
-      <c r="AK109" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-3.7567457055565356E-2</v>
+        <v>3.3780915064045305E-2</v>
       </c>
       <c r="AL109" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.32111695325986439</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.37167726638456144</v>
       </c>
     </row>
     <row r="110" spans="25:38" x14ac:dyDescent="0.25">
@@ -5388,7 +5622,7 @@
         <v>46</v>
       </c>
       <c r="Z110" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.10861069729595417</v>
       </c>
       <c r="AG110">
         <v>20</v>
@@ -5397,20 +5631,20 @@
         <v>1</v>
       </c>
       <c r="AI110" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>1.0179210039081191E-2</v>
+      </c>
+      <c r="AJ110" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AK110" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>-4.8886798044991277E-2</v>
-      </c>
-      <c r="AJ110" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.9511132019550087</v>
-      </c>
-      <c r="AK110" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-2.1778865952794702E-2</v>
+        <v>-3.3767417604063807E-2</v>
       </c>
       <c r="AL110" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.92933433600221405</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0.96623258239593623</v>
       </c>
     </row>
     <row r="111" spans="25:38" x14ac:dyDescent="0.25">
@@ -5418,7 +5652,7 @@
         <v>47</v>
       </c>
       <c r="Z111" t="str">
-        <v xml:space="preserve"> 0.6466465957242477</v>
+        <v xml:space="preserve"> 0.29557917692469254</v>
       </c>
       <c r="AG111">
         <v>21</v>
@@ -5427,20 +5661,20 @@
         <v>1</v>
       </c>
       <c r="AI111" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>-8.5083676334248085E-3</v>
+      </c>
+      <c r="AJ111" s="5">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.99149163236657523</v>
+      </c>
+      <c r="AK111" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>3.2016327268814343E-2</v>
-      </c>
-      <c r="AJ111" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="AK111" s="5">
-        <f t="shared" ca="1" si="1"/>
-        <v>-8.6431977468544446E-3</v>
+        <v>2.9221443236142425E-2</v>
       </c>
       <c r="AL111" s="5">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.9913568022531456</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="25:38" x14ac:dyDescent="0.25">
@@ -5448,7 +5682,7 @@
         <v>48</v>
       </c>
       <c r="Z112" t="str">
-        <v xml:space="preserve"> 1.0</v>
+        <v xml:space="preserve"> 0.8715150786731626</v>
       </c>
       <c r="AG112">
         <v>22</v>
@@ -5464,7 +5698,7 @@
         <v>49</v>
       </c>
       <c r="Z113" t="str">
-        <v xml:space="preserve"> 0.5074274005848062</v>
+        <v xml:space="preserve"> 0.839398210617237</v>
       </c>
     </row>
     <row r="114" spans="25:26" x14ac:dyDescent="0.25">
@@ -5472,7 +5706,7 @@
         <v>50</v>
       </c>
       <c r="Z114" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.6870816863298209</v>
       </c>
     </row>
     <row r="115" spans="25:26" x14ac:dyDescent="0.25">
@@ -5480,7 +5714,7 @@
         <v>51</v>
       </c>
       <c r="Z115" t="str">
-        <v xml:space="preserve"> 0.14289177800553857</v>
+        <v xml:space="preserve"> 0.6557872328730052</v>
       </c>
     </row>
     <row r="116" spans="25:26" x14ac:dyDescent="0.25">
@@ -5488,7 +5722,7 @@
         <v>52</v>
       </c>
       <c r="Z116" t="str">
-        <v xml:space="preserve"> 0.5623716489913057</v>
+        <v xml:space="preserve"> 0.13697399763482626</v>
       </c>
     </row>
     <row r="117" spans="25:26" x14ac:dyDescent="0.25">
@@ -5496,7 +5730,7 @@
         <v>53</v>
       </c>
       <c r="Z117" t="str">
-        <v xml:space="preserve"> 0.24690025994053244</v>
+        <v xml:space="preserve"> 0.16569205613001692</v>
       </c>
     </row>
     <row r="118" spans="25:26" x14ac:dyDescent="0.25">
@@ -5504,7 +5738,7 @@
         <v>54</v>
       </c>
       <c r="Z118" t="str">
-        <v xml:space="preserve"> 0.0</v>
+        <v xml:space="preserve"> 0.7745538427122949</v>
       </c>
     </row>
     <row r="119" spans="25:26" x14ac:dyDescent="0.25">
@@ -5512,7 +5746,7 @@
         <v>55</v>
       </c>
       <c r="Z119" t="str">
-        <v xml:space="preserve"> 0.30105336034734864</v>
+        <v xml:space="preserve"> 0.2968141695339541</v>
       </c>
     </row>
     <row r="120" spans="25:26" x14ac:dyDescent="0.25">
@@ -5520,68 +5754,46 @@
         <v>56</v>
       </c>
       <c r="Z120" t="str">
-        <v xml:space="preserve"> 0.9065068994520135</v>
+        <v xml:space="preserve"> 1.5314411976433369</v>
       </c>
     </row>
     <row r="121" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y121">
         <v>57</v>
       </c>
-      <c r="Z121" t="str">
-        <v xml:space="preserve"> 0.0</v>
-      </c>
     </row>
     <row r="122" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y122">
         <v>58</v>
       </c>
-      <c r="Z122" t="str">
-        <v xml:space="preserve"> 0.26961343445188857</v>
-      </c>
     </row>
     <row r="123" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y123">
         <v>59</v>
       </c>
-      <c r="Z123" t="str">
-        <v xml:space="preserve"> 0.5041212070306388</v>
-      </c>
     </row>
     <row r="124" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y124">
         <v>60</v>
       </c>
-      <c r="Z124" t="str">
-        <v xml:space="preserve"> 0.48225812616933666</v>
-      </c>
     </row>
     <row r="125" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y125">
         <v>61</v>
       </c>
-      <c r="Z125" t="str">
-        <v xml:space="preserve"> 0.4244568258071524</v>
-      </c>
     </row>
     <row r="126" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y126">
         <v>62</v>
       </c>
-      <c r="Z126" t="str">
-        <v xml:space="preserve"> 0.5040165654971762</v>
-      </c>
     </row>
     <row r="127" spans="25:26" x14ac:dyDescent="0.25">
       <c r="Y127">
         <v>63</v>
       </c>
-      <c r="Z127" t="str">
-        <v xml:space="preserve"> 0.31869428836394775</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="O29:W30"/>
     <mergeCell ref="C29:K30"/>
     <mergeCell ref="AA29:AI30"/>
     <mergeCell ref="AY29:BG30"/>
@@ -5590,6 +5802,7 @@
     <mergeCell ref="AM29:AU30"/>
     <mergeCell ref="AB1:AJ2"/>
     <mergeCell ref="AN1:AV2"/>
+    <mergeCell ref="O29:W30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="9">
@@ -5608,7 +5821,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE9BAA-8977-4D22-B011-D77539E65F64}">
-  <dimension ref="A1:AY19"/>
+  <dimension ref="A1:BZ41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -5618,23 +5831,27 @@
     <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.140625" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" customWidth="1"/>
     <col min="25" max="25" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="39" width="14.7109375" customWidth="1"/>
+    <col min="43" max="43" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="53" max="66" width="14.7109375" customWidth="1"/>
+    <col min="68" max="69" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:78" x14ac:dyDescent="0.25">
       <c r="B1" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
@@ -5647,7 +5864,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="N1" s="8">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O1" s="8"/>
       <c r="P1" s="8"/>
@@ -5660,8 +5877,9 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
-      <c r="AA1" s="8">
-        <v>28</v>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="8" t="s">
+        <v>103</v>
       </c>
       <c r="AB1" s="8"/>
       <c r="AC1" s="8"/>
@@ -5674,18 +5892,49 @@
       <c r="AJ1" s="1"/>
       <c r="AK1" s="1"/>
       <c r="AL1" s="1"/>
-      <c r="AN1" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AO1" s="8"/>
+      <c r="AM1" s="1"/>
+      <c r="AO1" s="8">
+        <v>28</v>
+      </c>
       <c r="AP1" s="8"/>
       <c r="AQ1" s="8"/>
       <c r="AR1" s="8"/>
       <c r="AS1" s="8"/>
       <c r="AT1" s="8"/>
       <c r="AU1" s="8"/>
-    </row>
-    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="AV1" s="8"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="BC1" s="8"/>
+      <c r="BD1" s="8"/>
+      <c r="BE1" s="8"/>
+      <c r="BF1" s="8"/>
+      <c r="BG1" s="8"/>
+      <c r="BH1" s="8"/>
+      <c r="BI1" s="8"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="BP1" s="8"/>
+      <c r="BQ1" s="8"/>
+      <c r="BR1" s="8"/>
+      <c r="BS1" s="8"/>
+      <c r="BT1" s="8"/>
+      <c r="BU1" s="8"/>
+      <c r="BV1" s="8"/>
+    </row>
+    <row r="2" spans="1:78" x14ac:dyDescent="0.25">
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -5709,6 +5958,7 @@
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
       <c r="AA2" s="8"/>
       <c r="AB2" s="8"/>
       <c r="AC2" s="8"/>
@@ -5721,7 +5971,7 @@
       <c r="AJ2" s="1"/>
       <c r="AK2" s="1"/>
       <c r="AL2" s="1"/>
-      <c r="AN2" s="8"/>
+      <c r="AM2" s="1"/>
       <c r="AO2" s="8"/>
       <c r="AP2" s="8"/>
       <c r="AQ2" s="8"/>
@@ -5729,10 +5979,37 @@
       <c r="AS2" s="8"/>
       <c r="AT2" s="8"/>
       <c r="AU2" s="8"/>
-    </row>
-    <row r="3" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="AV2" s="8"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="8"/>
+      <c r="BC2" s="8"/>
+      <c r="BD2" s="8"/>
+      <c r="BE2" s="8"/>
+      <c r="BF2" s="8"/>
+      <c r="BG2" s="8"/>
+      <c r="BH2" s="8"/>
+      <c r="BI2" s="8"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="8"/>
+      <c r="BP2" s="8"/>
+      <c r="BQ2" s="8"/>
+      <c r="BR2" s="8"/>
+      <c r="BS2" s="8"/>
+      <c r="BT2" s="8"/>
+      <c r="BU2" s="8"/>
+      <c r="BV2" s="8"/>
+    </row>
+    <row r="3" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
         <v>61</v>
@@ -5744,19 +6021,19 @@
         <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H3" t="s">
         <v>64</v>
       </c>
       <c r="N3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O3" t="s">
         <v>61</v>
@@ -5768,19 +6045,19 @@
         <v>63</v>
       </c>
       <c r="R3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U3" t="s">
         <v>64</v>
       </c>
       <c r="AA3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="AB3" t="s">
         <v>61</v>
@@ -5792,63 +6069,135 @@
         <v>63</v>
       </c>
       <c r="AE3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="AF3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="AG3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AH3" t="s">
         <v>64</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AI3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>62</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AS3" t="s">
         <v>68</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AT3" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>66</v>
+      </c>
+      <c r="BC3" t="s">
         <v>61</v>
       </c>
-      <c r="AP3" t="s">
+      <c r="BD3" t="s">
         <v>62</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="BE3" t="s">
         <v>63</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="BF3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>69</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>65</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>64</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>71</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>72</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>73</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>74</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP3" t="s">
+        <v>61</v>
+      </c>
+      <c r="BQ3" t="s">
+        <v>62</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>63</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT3" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU3" t="s">
+        <v>65</v>
+      </c>
+      <c r="BV3" t="s">
+        <v>64</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>71</v>
+      </c>
+      <c r="BX3" t="s">
+        <v>72</v>
+      </c>
+      <c r="BY3" t="s">
+        <v>73</v>
+      </c>
+      <c r="BZ3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
         <v>70</v>
       </c>
-      <c r="AS3" t="s">
-        <v>71</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>64</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX3" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" t="s">
-        <v>66</v>
+      <c r="C4">
+        <v>63</v>
       </c>
       <c r="D4">
         <v>18000</v>
@@ -5869,13 +6218,13 @@
         <v>8136</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O4" t="s">
-        <v>65</v>
-      </c>
-      <c r="P4" t="s">
-        <v>66</v>
+        <v>70</v>
+      </c>
+      <c r="P4">
+        <v>63</v>
       </c>
       <c r="Q4">
         <v>18000</v>
@@ -5896,63 +6245,161 @@
         <v>8136</v>
       </c>
       <c r="AA4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>65</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="AD4">
         <v>18000</v>
       </c>
-      <c r="AE4" s="5">
+      <c r="AE4">
         <f>AG4/AD4</f>
-        <v>0.53833333333333333</v>
+        <v>0</v>
       </c>
       <c r="AF4">
         <f>1-AE4</f>
-        <v>0.46166666666666667</v>
-      </c>
-      <c r="AG4">
-        <v>9690</v>
+        <v>1</v>
       </c>
       <c r="AH4">
         <f>AD4-AG4</f>
+        <v>18000</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ4">
+        <v>28</v>
+      </c>
+      <c r="AR4">
+        <v>18000</v>
+      </c>
+      <c r="AS4" s="5">
+        <f>AU4/AR4</f>
+        <v>0.53833333333333333</v>
+      </c>
+      <c r="AT4">
+        <f>1-AS4</f>
+        <v>0.46166666666666667</v>
+      </c>
+      <c r="AU4">
+        <v>9690</v>
+      </c>
+      <c r="AV4">
+        <f>AR4-AU4</f>
         <v>8310</v>
       </c>
-      <c r="AN4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>65</v>
-      </c>
-      <c r="AP4" t="s">
-        <v>75</v>
-      </c>
-      <c r="AQ4">
+      <c r="BB4" t="s">
+        <v>67</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>70</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>79</v>
+      </c>
+      <c r="BE4">
         <v>18000</v>
       </c>
-      <c r="AR4">
-        <f>AT4/AQ4</f>
+      <c r="BF4">
+        <f>BH4/BE4</f>
+        <v>0.998</v>
+      </c>
+      <c r="BG4">
+        <f>1-BF4</f>
+        <v>2.0000000000000018E-3</v>
+      </c>
+      <c r="BH4">
+        <v>17964</v>
+      </c>
+      <c r="BI4">
+        <f>BE4-BH4</f>
+        <v>36</v>
+      </c>
+      <c r="BJ4">
+        <v>14.3</v>
+      </c>
+      <c r="BK4">
+        <v>16.8</v>
+      </c>
+      <c r="BL4">
+        <v>27.42</v>
+      </c>
+      <c r="BM4">
+        <v>16.32</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>67</v>
+      </c>
+      <c r="BP4" t="s">
+        <v>70</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>109</v>
+      </c>
+      <c r="BR4">
+        <v>18000</v>
+      </c>
+      <c r="BS4">
+        <f>BU4/BR4</f>
         <v>0.41111111111111109</v>
       </c>
-      <c r="AS4" s="5">
-        <f>1-AR4</f>
+      <c r="BT4" s="5">
+        <f>1-BS4</f>
         <v>0.58888888888888891</v>
       </c>
-      <c r="AT4">
+      <c r="BU4">
         <v>7400</v>
       </c>
-      <c r="AU4">
-        <f>AQ4-AT4</f>
+      <c r="BV4">
+        <f>BR4-BU4</f>
         <v>10600</v>
       </c>
     </row>
-    <row r="6" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="BB5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>70</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BE5">
+        <v>18000</v>
+      </c>
+      <c r="BF5">
+        <f>BH5/BE5</f>
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="BG5">
+        <f>1-BF5</f>
+        <v>0.28500000000000003</v>
+      </c>
+      <c r="BH5">
+        <v>12870</v>
+      </c>
+      <c r="BI5">
+        <f>BE5-BH5</f>
+        <v>5130</v>
+      </c>
+      <c r="BJ5">
+        <v>19.5</v>
+      </c>
+      <c r="BK5">
+        <v>22.2</v>
+      </c>
+      <c r="BL5">
+        <v>22.6</v>
+      </c>
+      <c r="BM5">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
         <v>61</v>
@@ -5964,19 +6411,19 @@
         <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
         <v>64</v>
       </c>
       <c r="N6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O6" t="s">
         <v>61</v>
@@ -5988,19 +6435,19 @@
         <v>63</v>
       </c>
       <c r="R6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="S6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U6" t="s">
         <v>64</v>
       </c>
       <c r="AA6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="AB6" t="s">
         <v>61</v>
@@ -6012,75 +6459,111 @@
         <v>63</v>
       </c>
       <c r="AE6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="AF6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="AG6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AH6" t="s">
         <v>64</v>
       </c>
       <c r="AI6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="AJ6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AK6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AL6" t="s">
-        <v>79</v>
-      </c>
-      <c r="AN6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>62</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AS6" t="s">
         <v>68</v>
       </c>
-      <c r="AO6" t="s">
+      <c r="AT6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>71</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>72</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>74</v>
+      </c>
+      <c r="BO6" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP6" t="s">
         <v>61</v>
       </c>
-      <c r="AP6" t="s">
+      <c r="BQ6" t="s">
         <v>62</v>
       </c>
-      <c r="AQ6" t="s">
+      <c r="BR6" t="s">
         <v>63</v>
       </c>
-      <c r="AR6" t="s">
+      <c r="BS6" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT6" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU6" t="s">
+        <v>65</v>
+      </c>
+      <c r="BV6" t="s">
+        <v>64</v>
+      </c>
+      <c r="BW6" t="s">
+        <v>71</v>
+      </c>
+      <c r="BX6" t="s">
+        <v>72</v>
+      </c>
+      <c r="BY6" t="s">
+        <v>73</v>
+      </c>
+      <c r="BZ6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" t="s">
         <v>70</v>
       </c>
-      <c r="AS6" t="s">
-        <v>71</v>
-      </c>
-      <c r="AT6" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU6" t="s">
-        <v>64</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>76</v>
-      </c>
-      <c r="AW6" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX6" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" t="s">
-        <v>72</v>
+      <c r="C7">
+        <v>28</v>
       </c>
       <c r="D7">
         <v>18000</v>
@@ -6101,13 +6584,13 @@
         <v>8310</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
-      </c>
-      <c r="O7" t="s">
-        <v>66</v>
-      </c>
-      <c r="P7" t="s">
-        <v>72</v>
+        <v>67</v>
+      </c>
+      <c r="O7">
+        <v>63</v>
+      </c>
+      <c r="P7">
+        <v>28</v>
       </c>
       <c r="Q7">
         <v>18000</v>
@@ -6128,75 +6611,93 @@
         <v>9487</v>
       </c>
       <c r="AA7" t="s">
-        <v>69</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="AD7">
         <v>18000</v>
       </c>
       <c r="AE7">
         <f>AG7/AD7</f>
-        <v>0.47294444444444445</v>
+        <v>0</v>
       </c>
       <c r="AF7">
         <f>1-AE7</f>
-        <v>0.52705555555555561</v>
-      </c>
-      <c r="AG7">
-        <v>8513</v>
+        <v>1</v>
       </c>
       <c r="AH7">
         <f>AD7-AG7</f>
+        <v>18000</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP7">
+        <v>63</v>
+      </c>
+      <c r="AQ7">
+        <v>28</v>
+      </c>
+      <c r="AR7">
+        <v>18000</v>
+      </c>
+      <c r="AS7">
+        <f>AU7/AR7</f>
+        <v>0.47294444444444445</v>
+      </c>
+      <c r="AT7">
+        <f>1-AS7</f>
+        <v>0.52705555555555561</v>
+      </c>
+      <c r="AU7">
+        <v>8513</v>
+      </c>
+      <c r="AV7">
+        <f>AR7-AU7</f>
         <v>9487</v>
       </c>
-      <c r="AN7" t="s">
-        <v>69</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>65</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>75</v>
-      </c>
-      <c r="AQ7">
+      <c r="BO7" t="s">
+        <v>67</v>
+      </c>
+      <c r="BP7" t="s">
+        <v>70</v>
+      </c>
+      <c r="BQ7" t="s">
+        <v>109</v>
+      </c>
+      <c r="BR7">
         <v>18000</v>
       </c>
-      <c r="AR7">
-        <f>AT7/AQ7</f>
+      <c r="BS7">
+        <f>BU7/BR7</f>
         <v>0.4097777777777778</v>
       </c>
-      <c r="AS7" s="5">
-        <f>1-AR7</f>
+      <c r="BT7" s="5">
+        <f>1-BS7</f>
         <v>0.5902222222222222</v>
       </c>
-      <c r="AT7">
+      <c r="BU7">
         <v>7376</v>
       </c>
-      <c r="AU7">
-        <f>AQ7-AT7</f>
+      <c r="BV7">
+        <f>BR7-BU7</f>
         <v>10624</v>
       </c>
-      <c r="AV7">
+      <c r="BW7">
         <v>20.25</v>
       </c>
-      <c r="AW7">
+      <c r="BX7">
         <v>19.59</v>
       </c>
-      <c r="AX7">
+      <c r="BY7">
         <v>18.62</v>
       </c>
-      <c r="AY7">
+      <c r="BZ7">
         <v>18.809999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
         <v>61</v>
@@ -6208,19 +6709,19 @@
         <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H9" t="s">
         <v>64</v>
       </c>
       <c r="N9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O9" t="s">
         <v>61</v>
@@ -6232,75 +6733,111 @@
         <v>63</v>
       </c>
       <c r="R9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="S9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U9" t="s">
         <v>64</v>
       </c>
       <c r="V9" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="W9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="X9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Y9" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>66</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>62</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AS9" t="s">
         <v>68</v>
       </c>
-      <c r="AB9" t="s">
+      <c r="AT9" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU9" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV9" t="s">
+        <v>64</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>71</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>72</v>
+      </c>
+      <c r="AY9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ9" t="s">
+        <v>74</v>
+      </c>
+      <c r="BO9" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP9" t="s">
         <v>61</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="BQ9" t="s">
         <v>62</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="BR9" t="s">
         <v>63</v>
       </c>
-      <c r="AE9" t="s">
+      <c r="BS9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT9" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU9" t="s">
+        <v>65</v>
+      </c>
+      <c r="BV9" t="s">
+        <v>64</v>
+      </c>
+      <c r="BW9" t="s">
+        <v>71</v>
+      </c>
+      <c r="BX9" t="s">
+        <v>72</v>
+      </c>
+      <c r="BY9" t="s">
+        <v>73</v>
+      </c>
+      <c r="BZ9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" t="s">
         <v>70</v>
       </c>
-      <c r="AF9" t="s">
-        <v>71</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH9" t="s">
-        <v>64</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>76</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AK9" t="s">
-        <v>78</v>
-      </c>
-      <c r="AL9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" t="s">
-        <v>65</v>
-      </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="D10">
         <v>18000</v>
@@ -6321,13 +6858,13 @@
         <v>10600</v>
       </c>
       <c r="N10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O10" t="s">
-        <v>65</v>
-      </c>
-      <c r="P10" t="s">
-        <v>66</v>
+        <v>70</v>
+      </c>
+      <c r="P10">
+        <v>63</v>
       </c>
       <c r="Q10">
         <v>18000</v>
@@ -6359,49 +6896,74 @@
       <c r="Y10">
         <v>18.14</v>
       </c>
-      <c r="AA10" t="s">
-        <v>69</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>65</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>72</v>
-      </c>
-      <c r="AD10">
+      <c r="AO10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ10">
+        <v>28</v>
+      </c>
+      <c r="AR10">
         <v>18000</v>
       </c>
-      <c r="AE10" s="5">
-        <f>AG10/AD10</f>
+      <c r="AS10" s="5">
+        <f>AU10/AR10</f>
         <v>0.53466666666666662</v>
       </c>
-      <c r="AF10">
-        <f>1-AE10</f>
+      <c r="AT10">
+        <f>1-AS10</f>
         <v>0.46533333333333338</v>
       </c>
-      <c r="AG10">
+      <c r="AU10">
         <v>9624</v>
       </c>
-      <c r="AH10">
-        <f>AD10-AG10</f>
+      <c r="AV10">
+        <f>AR10-AU10</f>
         <v>8376</v>
       </c>
-      <c r="AI10">
+      <c r="AW10">
         <v>19.39</v>
       </c>
-      <c r="AJ10">
+      <c r="AX10">
         <v>18.7</v>
       </c>
-      <c r="AK10">
+      <c r="AY10">
         <v>17.73</v>
       </c>
-      <c r="AL10">
+      <c r="AZ10">
         <v>18.62</v>
       </c>
-    </row>
-    <row r="12" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="BF10" s="5"/>
+      <c r="BO10" t="s">
+        <v>67</v>
+      </c>
+      <c r="BP10" t="s">
+        <v>110</v>
+      </c>
+      <c r="BQ10" t="s">
+        <v>109</v>
+      </c>
+      <c r="BR10">
+        <v>18000</v>
+      </c>
+      <c r="BS10">
+        <f>BU10/BR10</f>
+        <v>0</v>
+      </c>
+      <c r="BT10" s="5">
+        <f>1-BS10</f>
+        <v>1</v>
+      </c>
+      <c r="BV10">
+        <f>BR10-BU10</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
         <v>61</v>
@@ -6413,39 +6975,39 @@
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
         <v>64</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J12" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:51" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" t="s">
-        <v>66</v>
+        <v>70</v>
+      </c>
+      <c r="C13">
+        <v>63</v>
       </c>
       <c r="D13">
         <v>18000</v>
@@ -6478,9 +7040,9 @@
         <v>18.14</v>
       </c>
     </row>
-    <row r="15" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
         <v>61</v>
@@ -6492,39 +7054,39 @@
         <v>63</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H15" t="s">
         <v>64</v>
       </c>
       <c r="I15" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J15" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L15" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" t="s">
-        <v>72</v>
+        <v>70</v>
+      </c>
+      <c r="C16">
+        <v>28</v>
       </c>
       <c r="D16">
         <v>18000</v>
@@ -6559,7 +7121,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
         <v>61</v>
@@ -6571,39 +7133,39 @@
         <v>63</v>
       </c>
       <c r="E18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H18" t="s">
         <v>64</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J18" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L18" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="D19">
         <v>18000</v>
@@ -6636,12 +7198,151 @@
         <v>18.809999999999999</v>
       </c>
     </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" t="s">
+        <v>64</v>
+      </c>
+      <c r="I21" t="s">
+        <v>71</v>
+      </c>
+      <c r="J21" t="s">
+        <v>72</v>
+      </c>
+      <c r="K21" t="s">
+        <v>73</v>
+      </c>
+      <c r="L21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22">
+        <v>18000</v>
+      </c>
+      <c r="E22">
+        <f>G22/D22</f>
+        <v>0.998</v>
+      </c>
+      <c r="F22">
+        <f>1-E22</f>
+        <v>2.0000000000000018E-3</v>
+      </c>
+      <c r="G22">
+        <v>17964</v>
+      </c>
+      <c r="H22">
+        <f>D22-G22</f>
+        <v>36</v>
+      </c>
+      <c r="I22">
+        <v>14.3</v>
+      </c>
+      <c r="J22">
+        <v>16.8</v>
+      </c>
+      <c r="K22">
+        <v>27.42</v>
+      </c>
+      <c r="L22">
+        <v>16.32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" t="s">
+        <v>68</v>
+      </c>
+      <c r="F40" t="s">
+        <v>69</v>
+      </c>
+      <c r="G40" t="s">
+        <v>65</v>
+      </c>
+      <c r="H40" t="s">
+        <v>64</v>
+      </c>
+      <c r="I40" t="s">
+        <v>71</v>
+      </c>
+      <c r="J40" t="s">
+        <v>72</v>
+      </c>
+      <c r="K40" t="s">
+        <v>73</v>
+      </c>
+      <c r="L40" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>67</v>
+      </c>
+      <c r="D41">
+        <v>18000</v>
+      </c>
+      <c r="E41">
+        <f>G41/D41</f>
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <f>1-E41</f>
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <f>D41-G41</f>
+        <v>18000</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="B1:H2"/>
     <mergeCell ref="N1:U2"/>
+    <mergeCell ref="AO1:AV2"/>
+    <mergeCell ref="BO1:BV2"/>
     <mergeCell ref="AA1:AH2"/>
-    <mergeCell ref="AN1:AU2"/>
+    <mergeCell ref="BB1:BI2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update opponents list every X iteration
</commit_message>
<xml_diff>
--- a/core-extensions/SabberStoneCoreAi/my_results/experiments-analysis.xlsx
+++ b/core-extensions/SabberStoneCoreAi/my_results/experiments-analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pics_Movies\vids\PWr\Sem10\magisterka\SabberStone\core-extensions\SabberStoneCoreAi\my_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA6A0C8-CC1D-470E-A0C4-B05CC103F9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3070984D-88A4-4B93-9388-70DC1E181FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="3900" windowWidth="28800" windowHeight="15885" activeTab="1" xr2:uid="{23FC15A1-DE11-4199-B1D8-4DE8B55B0A24}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="1" xr2:uid="{23FC15A1-DE11-4199-B1D8-4DE8B55B0A24}"/>
   </bookViews>
   <sheets>
     <sheet name="Weights" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="125">
   <si>
     <t>Hero Health Reduced</t>
   </si>
@@ -427,10 +427,13 @@
     <t>pure-Shade</t>
   </si>
   <si>
-    <t>0.4091753041621535, 0.526987531425831, 0.07765675894938162, 0.004964104866896055, 0.6199393341507159, 0.7247614063773686, 0.45860226419395134, 0.15632117815261173, 0.40243406150630634, 0.963374090223104, 0.3005745081849112, 0.4181724138063309, 0.217602282503368, 0.05208753079827609, 0.18864788546957187, 0.3360597767270444, 0.06567990706602098, 0.1747001120497397, 0.5085210161287994, 0.21394113718953117, 0.7389415568300491</t>
-  </si>
-  <si>
-    <t>0.409175#0.526988#0.077657#0.004964#0.619939#0.724761#0.458602#0.156321#0.402434#0.963374#0.300575#0.418172#0.217602#0.052088#0.188648#0.33606#0.06568#0.1747#0.508521#0.213941#0.738942</t>
+    <t>pure-Shade-csv-change</t>
+  </si>
+  <si>
+    <t>0.4679608226343523, 0.9362630083244707, 0.045734449308683464, 0.12002048293538281, 0.9753029321700649, 0.9216730696463928, 0.2557964891936836, 0.027180268139501307, 0.9210008983160494, 0.7570458084288632, 0.18026046331816964, 0.08627965223235323, 0.820517756196796, 0.3505850348410258, 0.09511029639349017, 0.4095055766044159, 0.9984030094579434, 0.8897979995460684, 0.08827405019913738, 0.3570230554028749, 0.5880257881917569</t>
+  </si>
+  <si>
+    <t>0.467960822634352#0.93626300832447#0.0457344493086834#0.120020482935382#0.975302932170064#0.921673069646392#0.255796489193683#0.0271802681395013#0.921000898316049#0.757045808428863#0.180260463318169#0.0862796522323532#0.820517756196796#0.350585034841025#0.0951102963934901#0.409505576604415#0.998403009457943#0.889797999546068#0.0882740501991373#0.357023055402874#0.588025788191756</t>
   </si>
 </sst>
 </file>
@@ -516,7 +519,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -527,14 +530,12 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,8 +590,8 @@
     <tableColumn id="1" xr3:uid="{D55A2F50-BBE7-4C22-9C9C-3852D667EA62}" name="NUM_GAMES"/>
     <tableColumn id="2" xr3:uid="{D1FBD886-6DEC-4555-85EE-6E978CA095FB}" name="POP_SIZE"/>
     <tableColumn id="3" xr3:uid="{E7086050-75AA-4B8A-8F23-5307D7D87E54}" name="MAX_EVALUATIONS"/>
-    <tableColumn id="4" xr3:uid="{5706D084-1645-435D-8942-D533E099E7D5}" name="Max fitness" dataDxfId="2">
-      <calculatedColumnFormula>3*9*Table363511[[#This Row],[NUM_GAMES]]</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{5706D084-1645-435D-8942-D533E099E7D5}" name="Max fitness" dataDxfId="1">
+      <calculatedColumnFormula>BY32*(2*BZ32-1)*9</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{A7D12601-BF17-468C-8F22-2708F2D253B3}" name="Worst"/>
     <tableColumn id="6" xr3:uid="{4FDAF113-60D6-475F-9197-FD603D14B26E}" name="Best"/>
@@ -609,10 +610,10 @@
     <tableColumn id="1" xr3:uid="{E188DA55-F8ED-43CA-BF85-DA0D630AB557}" name="NUM_GAMES"/>
     <tableColumn id="2" xr3:uid="{129F20C9-39DF-4159-B851-0B89D53D54E9}" name="POP_SIZE"/>
     <tableColumn id="3" xr3:uid="{93D924ED-DA6A-4436-BEA0-C1A635CDB36A}" name="MAX_EVALUATIONS"/>
-    <tableColumn id="4" xr3:uid="{A02C2CDB-E9A9-4E69-8CEA-6F7E3FC9D952}" name="Max fitness" dataDxfId="1">
-      <calculatedColumnFormula>Table36351112[[#This Row],[NUM_GAMES]]*(Table36351112[[#This Row],[POP_SIZE]]-1)*9</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{A02C2CDB-E9A9-4E69-8CEA-6F7E3FC9D952}" name="Max fitness" dataDxfId="0">
+      <calculatedColumnFormula>BY32*(2*BZ32-1)*9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{ACC46462-3E6D-405B-99AE-C442AEAB28E3}" name="Worst" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{ACC46462-3E6D-405B-99AE-C442AEAB28E3}" name="Worst" dataDxfId="2">
       <calculatedColumnFormula>IF(Table36351112[[#This Row],[Max fitness]]&gt;0.1,"y","")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{3487042A-ED8B-42D5-938D-DF32EC17453D}" name="Best"/>
@@ -1144,51 +1145,52 @@
     <col min="67" max="67" width="12.85546875" customWidth="1"/>
     <col min="68" max="68" width="13.85546875" customWidth="1"/>
     <col min="87" max="87" width="15.5703125" customWidth="1"/>
+    <col min="103" max="103" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="26:48" hidden="1" x14ac:dyDescent="0.25">
-      <c r="AB1" s="8" t="s">
+      <c r="AB1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-      <c r="AH1" s="8"/>
-      <c r="AI1" s="8"/>
-      <c r="AJ1" s="8"/>
-      <c r="AN1" s="8" t="s">
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="10"/>
+      <c r="AH1" s="10"/>
+      <c r="AI1" s="10"/>
+      <c r="AJ1" s="10"/>
+      <c r="AN1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AO1" s="8"/>
-      <c r="AP1" s="8"/>
-      <c r="AQ1" s="8"/>
-      <c r="AR1" s="8"/>
-      <c r="AS1" s="8"/>
-      <c r="AT1" s="8"/>
-      <c r="AU1" s="8"/>
-      <c r="AV1" s="8"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="10"/>
+      <c r="AR1" s="10"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="10"/>
+      <c r="AU1" s="10"/>
+      <c r="AV1" s="10"/>
     </row>
     <row r="2" spans="26:48" hidden="1" x14ac:dyDescent="0.25">
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="8"/>
-      <c r="AD2" s="8"/>
-      <c r="AE2" s="8"/>
-      <c r="AF2" s="8"/>
-      <c r="AG2" s="8"/>
-      <c r="AH2" s="8"/>
-      <c r="AI2" s="8"/>
-      <c r="AJ2" s="8"/>
-      <c r="AN2" s="8"/>
-      <c r="AO2" s="8"/>
-      <c r="AP2" s="8"/>
-      <c r="AQ2" s="8"/>
-      <c r="AR2" s="8"/>
-      <c r="AS2" s="8"/>
-      <c r="AT2" s="8"/>
-      <c r="AU2" s="8"/>
-      <c r="AV2" s="8"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10"/>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="10"/>
+      <c r="AJ2" s="10"/>
+      <c r="AN2" s="10"/>
+      <c r="AO2" s="10"/>
+      <c r="AP2" s="10"/>
+      <c r="AQ2" s="10"/>
+      <c r="AR2" s="10"/>
+      <c r="AS2" s="10"/>
+      <c r="AT2" s="10"/>
+      <c r="AU2" s="10"/>
+      <c r="AV2" s="10"/>
     </row>
     <row r="3" spans="26:48" hidden="1" x14ac:dyDescent="0.25">
       <c r="AB3" t="s">
@@ -1870,192 +1872,192 @@
     <row r="27" spans="3:109" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="3:109" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="3:109" x14ac:dyDescent="0.25">
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
-      <c r="O29" s="8" t="s">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="O29" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="8"/>
-      <c r="S29" s="8"/>
-      <c r="T29" s="8"/>
-      <c r="U29" s="8"/>
-      <c r="V29" s="8"/>
-      <c r="W29" s="8"/>
-      <c r="AA29" s="8" t="s">
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="10"/>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10"/>
+      <c r="W29" s="10"/>
+      <c r="AA29" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="AB29" s="8"/>
-      <c r="AC29" s="8"/>
-      <c r="AD29" s="8"/>
-      <c r="AE29" s="8"/>
-      <c r="AF29" s="8"/>
-      <c r="AG29" s="8"/>
-      <c r="AH29" s="8"/>
-      <c r="AI29" s="8"/>
-      <c r="AM29" s="8" t="s">
+      <c r="AB29" s="10"/>
+      <c r="AC29" s="10"/>
+      <c r="AD29" s="10"/>
+      <c r="AE29" s="10"/>
+      <c r="AF29" s="10"/>
+      <c r="AG29" s="10"/>
+      <c r="AH29" s="10"/>
+      <c r="AI29" s="10"/>
+      <c r="AM29" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="AN29" s="8"/>
-      <c r="AO29" s="8"/>
-      <c r="AP29" s="8"/>
-      <c r="AQ29" s="8"/>
-      <c r="AR29" s="8"/>
-      <c r="AS29" s="8"/>
-      <c r="AT29" s="8"/>
-      <c r="AU29" s="8"/>
-      <c r="AY29" s="8" t="s">
+      <c r="AN29" s="10"/>
+      <c r="AO29" s="10"/>
+      <c r="AP29" s="10"/>
+      <c r="AQ29" s="10"/>
+      <c r="AR29" s="10"/>
+      <c r="AS29" s="10"/>
+      <c r="AT29" s="10"/>
+      <c r="AU29" s="10"/>
+      <c r="AY29" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="AZ29" s="8"/>
-      <c r="BA29" s="8"/>
-      <c r="BB29" s="8"/>
-      <c r="BC29" s="8"/>
-      <c r="BD29" s="8"/>
-      <c r="BE29" s="8"/>
-      <c r="BF29" s="8"/>
-      <c r="BG29" s="8"/>
-      <c r="BK29" s="8" t="s">
+      <c r="AZ29" s="10"/>
+      <c r="BA29" s="10"/>
+      <c r="BB29" s="10"/>
+      <c r="BC29" s="10"/>
+      <c r="BD29" s="10"/>
+      <c r="BE29" s="10"/>
+      <c r="BF29" s="10"/>
+      <c r="BG29" s="10"/>
+      <c r="BK29" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="BL29" s="8"/>
-      <c r="BM29" s="8"/>
-      <c r="BN29" s="8"/>
-      <c r="BO29" s="8"/>
-      <c r="BP29" s="8"/>
-      <c r="BQ29" s="8"/>
-      <c r="BR29" s="8"/>
-      <c r="BS29" s="8"/>
-      <c r="BT29" s="8"/>
-      <c r="BU29" s="8"/>
-      <c r="BY29" s="8" t="s">
+      <c r="BL29" s="10"/>
+      <c r="BM29" s="10"/>
+      <c r="BN29" s="10"/>
+      <c r="BO29" s="10"/>
+      <c r="BP29" s="10"/>
+      <c r="BQ29" s="10"/>
+      <c r="BR29" s="10"/>
+      <c r="BS29" s="10"/>
+      <c r="BT29" s="10"/>
+      <c r="BU29" s="10"/>
+      <c r="BY29" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="BZ29" s="8"/>
-      <c r="CA29" s="8"/>
-      <c r="CB29" s="8"/>
-      <c r="CC29" s="8"/>
-      <c r="CD29" s="8"/>
-      <c r="CE29" s="8"/>
-      <c r="CF29" s="8"/>
-      <c r="CG29" s="8"/>
-      <c r="CK29" s="8" t="s">
+      <c r="BZ29" s="10"/>
+      <c r="CA29" s="10"/>
+      <c r="CB29" s="10"/>
+      <c r="CC29" s="10"/>
+      <c r="CD29" s="10"/>
+      <c r="CE29" s="10"/>
+      <c r="CF29" s="10"/>
+      <c r="CG29" s="10"/>
+      <c r="CK29" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="CL29" s="8"/>
-      <c r="CM29" s="8"/>
-      <c r="CN29" s="8"/>
-      <c r="CO29" s="8"/>
-      <c r="CP29" s="8"/>
-      <c r="CQ29" s="8"/>
-      <c r="CR29" s="8"/>
-      <c r="CS29" s="8"/>
-      <c r="CW29" s="8" t="s">
+      <c r="CL29" s="10"/>
+      <c r="CM29" s="10"/>
+      <c r="CN29" s="10"/>
+      <c r="CO29" s="10"/>
+      <c r="CP29" s="10"/>
+      <c r="CQ29" s="10"/>
+      <c r="CR29" s="10"/>
+      <c r="CS29" s="10"/>
+      <c r="CW29" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="CX29" s="8"/>
-      <c r="CY29" s="8"/>
-      <c r="CZ29" s="8"/>
-      <c r="DA29" s="8"/>
-      <c r="DB29" s="8"/>
-      <c r="DC29" s="8"/>
-      <c r="DD29" s="8"/>
-      <c r="DE29" s="8"/>
+      <c r="CX29" s="10"/>
+      <c r="CY29" s="10"/>
+      <c r="CZ29" s="10"/>
+      <c r="DA29" s="10"/>
+      <c r="DB29" s="10"/>
+      <c r="DC29" s="10"/>
+      <c r="DD29" s="10"/>
+      <c r="DE29" s="10"/>
     </row>
     <row r="30" spans="3:109" x14ac:dyDescent="0.25">
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8"/>
-      <c r="S30" s="8"/>
-      <c r="T30" s="8"/>
-      <c r="U30" s="8"/>
-      <c r="V30" s="8"/>
-      <c r="W30" s="8"/>
-      <c r="AA30" s="8"/>
-      <c r="AB30" s="8"/>
-      <c r="AC30" s="8"/>
-      <c r="AD30" s="8"/>
-      <c r="AE30" s="8"/>
-      <c r="AF30" s="8"/>
-      <c r="AG30" s="8"/>
-      <c r="AH30" s="8"/>
-      <c r="AI30" s="8"/>
-      <c r="AM30" s="8"/>
-      <c r="AN30" s="8"/>
-      <c r="AO30" s="8"/>
-      <c r="AP30" s="8"/>
-      <c r="AQ30" s="8"/>
-      <c r="AR30" s="8"/>
-      <c r="AS30" s="8"/>
-      <c r="AT30" s="8"/>
-      <c r="AU30" s="8"/>
-      <c r="AY30" s="8"/>
-      <c r="AZ30" s="8"/>
-      <c r="BA30" s="8"/>
-      <c r="BB30" s="8"/>
-      <c r="BC30" s="8"/>
-      <c r="BD30" s="8"/>
-      <c r="BE30" s="8"/>
-      <c r="BF30" s="8"/>
-      <c r="BG30" s="8"/>
-      <c r="BK30" s="8"/>
-      <c r="BL30" s="8"/>
-      <c r="BM30" s="8"/>
-      <c r="BN30" s="8"/>
-      <c r="BO30" s="8"/>
-      <c r="BP30" s="8"/>
-      <c r="BQ30" s="8"/>
-      <c r="BR30" s="8"/>
-      <c r="BS30" s="8"/>
-      <c r="BT30" s="8"/>
-      <c r="BU30" s="8"/>
-      <c r="BY30" s="8"/>
-      <c r="BZ30" s="8"/>
-      <c r="CA30" s="8"/>
-      <c r="CB30" s="8"/>
-      <c r="CC30" s="8"/>
-      <c r="CD30" s="8"/>
-      <c r="CE30" s="8"/>
-      <c r="CF30" s="8"/>
-      <c r="CG30" s="8"/>
-      <c r="CK30" s="8"/>
-      <c r="CL30" s="8"/>
-      <c r="CM30" s="8"/>
-      <c r="CN30" s="8"/>
-      <c r="CO30" s="8"/>
-      <c r="CP30" s="8"/>
-      <c r="CQ30" s="8"/>
-      <c r="CR30" s="8"/>
-      <c r="CS30" s="8"/>
-      <c r="CW30" s="8"/>
-      <c r="CX30" s="8"/>
-      <c r="CY30" s="8"/>
-      <c r="CZ30" s="8"/>
-      <c r="DA30" s="8"/>
-      <c r="DB30" s="8"/>
-      <c r="DC30" s="8"/>
-      <c r="DD30" s="8"/>
-      <c r="DE30" s="8"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="AA30" s="10"/>
+      <c r="AB30" s="10"/>
+      <c r="AC30" s="10"/>
+      <c r="AD30" s="10"/>
+      <c r="AE30" s="10"/>
+      <c r="AF30" s="10"/>
+      <c r="AG30" s="10"/>
+      <c r="AH30" s="10"/>
+      <c r="AI30" s="10"/>
+      <c r="AM30" s="10"/>
+      <c r="AN30" s="10"/>
+      <c r="AO30" s="10"/>
+      <c r="AP30" s="10"/>
+      <c r="AQ30" s="10"/>
+      <c r="AR30" s="10"/>
+      <c r="AS30" s="10"/>
+      <c r="AT30" s="10"/>
+      <c r="AU30" s="10"/>
+      <c r="AY30" s="10"/>
+      <c r="AZ30" s="10"/>
+      <c r="BA30" s="10"/>
+      <c r="BB30" s="10"/>
+      <c r="BC30" s="10"/>
+      <c r="BD30" s="10"/>
+      <c r="BE30" s="10"/>
+      <c r="BF30" s="10"/>
+      <c r="BG30" s="10"/>
+      <c r="BK30" s="10"/>
+      <c r="BL30" s="10"/>
+      <c r="BM30" s="10"/>
+      <c r="BN30" s="10"/>
+      <c r="BO30" s="10"/>
+      <c r="BP30" s="10"/>
+      <c r="BQ30" s="10"/>
+      <c r="BR30" s="10"/>
+      <c r="BS30" s="10"/>
+      <c r="BT30" s="10"/>
+      <c r="BU30" s="10"/>
+      <c r="BY30" s="10"/>
+      <c r="BZ30" s="10"/>
+      <c r="CA30" s="10"/>
+      <c r="CB30" s="10"/>
+      <c r="CC30" s="10"/>
+      <c r="CD30" s="10"/>
+      <c r="CE30" s="10"/>
+      <c r="CF30" s="10"/>
+      <c r="CG30" s="10"/>
+      <c r="CK30" s="10"/>
+      <c r="CL30" s="10"/>
+      <c r="CM30" s="10"/>
+      <c r="CN30" s="10"/>
+      <c r="CO30" s="10"/>
+      <c r="CP30" s="10"/>
+      <c r="CQ30" s="10"/>
+      <c r="CR30" s="10"/>
+      <c r="CS30" s="10"/>
+      <c r="CW30" s="10"/>
+      <c r="CX30" s="10"/>
+      <c r="CY30" s="10"/>
+      <c r="CZ30" s="10"/>
+      <c r="DA30" s="10"/>
+      <c r="DB30" s="10"/>
+      <c r="DC30" s="10"/>
+      <c r="DD30" s="10"/>
+      <c r="DE30" s="10"/>
     </row>
     <row r="31" spans="3:109" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
@@ -2500,8 +2502,8 @@
         <v>200</v>
       </c>
       <c r="CN32">
-        <f>Table36351112[[#This Row],[NUM_GAMES]]*(Table36351112[[#This Row],[POP_SIZE]]-1)*9</f>
-        <v>504</v>
+        <f t="shared" ref="CN32:CN56" si="0">BY32*(2*BZ32-1)*9</f>
+        <v>1080</v>
       </c>
       <c r="CW32">
         <v>8</v>
@@ -2513,11 +2515,11 @@
         <v>200</v>
       </c>
       <c r="CZ32">
-        <f>7*9*Table363511[[#This Row],[NUM_GAMES]]</f>
-        <v>504</v>
-      </c>
-    </row>
-    <row r="33" spans="1:102" x14ac:dyDescent="0.25">
+        <f t="shared" ref="CZ32:CZ53" si="1">BY32*(2*BZ32-1)*9</f>
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="33" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -2655,15 +2657,15 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="CD33">
-        <f t="shared" ref="CD33:CF33" si="0">CD32/$AD$32</f>
+        <f t="shared" ref="CD33:CF33" si="2">CD32/$AD$32</f>
         <v>0.66574074074074074</v>
       </c>
       <c r="CE33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0.62962962962962965</v>
       </c>
       <c r="CF33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0.62129629629629635</v>
       </c>
       <c r="CI33" t="s">
@@ -2675,7 +2677,7 @@
       <c r="CK33">
         <v>0.79772286000000003</v>
       </c>
-      <c r="CL33" s="11">
+      <c r="CL33">
         <v>0.29200656000000003</v>
       </c>
       <c r="CU33" t="s">
@@ -2684,12 +2686,14 @@
       <c r="CV33">
         <v>1</v>
       </c>
-      <c r="CW33" s="11">
+      <c r="CW33">
         <v>0.40917530416215298</v>
       </c>
-      <c r="CX33" s="11"/>
-    </row>
-    <row r="34" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY33" s="11">
+        <v>0.46796082263435201</v>
+      </c>
+    </row>
+    <row r="34" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
@@ -2783,7 +2787,7 @@
       <c r="CK34">
         <v>0.64642785999999997</v>
       </c>
-      <c r="CL34" s="11">
+      <c r="CL34">
         <v>0.98765521999999994</v>
       </c>
       <c r="CU34" t="s">
@@ -2792,12 +2796,14 @@
       <c r="CV34">
         <v>2</v>
       </c>
-      <c r="CW34" s="11">
+      <c r="CW34">
         <v>0.52698753142583099</v>
       </c>
-      <c r="CX34" s="11"/>
-    </row>
-    <row r="35" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY34" s="11">
+        <v>0.93626300832446996</v>
+      </c>
+    </row>
+    <row r="35" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -2891,7 +2897,7 @@
       <c r="CK35">
         <v>0.36333969999999999</v>
       </c>
-      <c r="CL35" s="11">
+      <c r="CL35">
         <v>2.0412759999999999E-2</v>
       </c>
       <c r="CU35" t="s">
@@ -2900,12 +2906,14 @@
       <c r="CV35">
         <v>3</v>
       </c>
-      <c r="CW35" s="11">
+      <c r="CW35">
         <v>7.7656758949381594E-2</v>
       </c>
-      <c r="CX35" s="11"/>
-    </row>
-    <row r="36" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY35" s="11">
+        <v>4.5734449308683402E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -2999,7 +3007,7 @@
       <c r="CK36">
         <v>0.78405817</v>
       </c>
-      <c r="CL36" s="11">
+      <c r="CL36">
         <v>0.63498946000000001</v>
       </c>
       <c r="CU36" t="s">
@@ -3008,12 +3016,14 @@
       <c r="CV36">
         <v>4</v>
       </c>
-      <c r="CW36" s="11">
+      <c r="CW36">
         <v>4.9641048668960502E-3</v>
       </c>
-      <c r="CX36" s="11"/>
-    </row>
-    <row r="37" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY36" s="11">
+        <v>0.12002048293538201</v>
+      </c>
+    </row>
+    <row r="37" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -3107,7 +3117,7 @@
       <c r="CK37">
         <v>0.53132201000000001</v>
       </c>
-      <c r="CL37" s="11">
+      <c r="CL37">
         <v>0.74946424</v>
       </c>
       <c r="CU37" t="s">
@@ -3116,12 +3126,14 @@
       <c r="CV37">
         <v>5</v>
       </c>
-      <c r="CW37" s="11">
+      <c r="CW37">
         <v>0.619939334150715</v>
       </c>
-      <c r="CX37" s="11"/>
-    </row>
-    <row r="38" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY37" s="11">
+        <v>0.97530293217006403</v>
+      </c>
+    </row>
+    <row r="38" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -3215,7 +3227,7 @@
       <c r="CK38">
         <v>0.70726014000000004</v>
       </c>
-      <c r="CL38" s="11">
+      <c r="CL38">
         <v>0.94758803999999996</v>
       </c>
       <c r="CU38" t="s">
@@ -3224,12 +3236,14 @@
       <c r="CV38">
         <v>6</v>
       </c>
-      <c r="CW38" s="11">
+      <c r="CW38">
         <v>0.72476140637736797</v>
       </c>
-      <c r="CX38" s="11"/>
-    </row>
-    <row r="39" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY38" s="11">
+        <v>0.92167306964639195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -3323,7 +3337,7 @@
       <c r="CK39">
         <v>0.37291523999999998</v>
       </c>
-      <c r="CL39" s="11">
+      <c r="CL39">
         <v>0.47603055999999999</v>
       </c>
       <c r="CU39" t="s">
@@ -3332,12 +3346,14 @@
       <c r="CV39">
         <v>7</v>
       </c>
-      <c r="CW39" s="11">
+      <c r="CW39">
         <v>0.458602264193951</v>
       </c>
-      <c r="CX39" s="11"/>
-    </row>
-    <row r="40" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY39" s="11">
+        <v>0.25579648919368297</v>
+      </c>
+    </row>
+    <row r="40" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>7</v>
       </c>
@@ -3431,7 +3447,7 @@
       <c r="CK40">
         <v>0.20189695999999999</v>
       </c>
-      <c r="CL40" s="11">
+      <c r="CL40">
         <v>5.9881980000000001E-2</v>
       </c>
       <c r="CU40" t="s">
@@ -3440,12 +3456,14 @@
       <c r="CV40">
         <v>8</v>
       </c>
-      <c r="CW40" s="11">
+      <c r="CW40">
         <v>0.15632117815261101</v>
       </c>
-      <c r="CX40" s="11"/>
-    </row>
-    <row r="41" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY40" s="11">
+        <v>2.71802681395013E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -3539,7 +3557,7 @@
       <c r="CK41">
         <v>7.0149279999999994E-2</v>
       </c>
-      <c r="CL41" s="11">
+      <c r="CL41">
         <v>0.40201173000000001</v>
       </c>
       <c r="CU41" t="s">
@@ -3548,12 +3566,14 @@
       <c r="CV41">
         <v>9</v>
       </c>
-      <c r="CW41" s="11">
+      <c r="CW41">
         <v>0.40243406150630601</v>
       </c>
-      <c r="CX41" s="11"/>
-    </row>
-    <row r="42" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY41" s="11">
+        <v>0.92100089831604903</v>
+      </c>
+    </row>
+    <row r="42" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -3647,7 +3667,7 @@
       <c r="CK42">
         <v>0.78355543999999999</v>
       </c>
-      <c r="CL42" s="11">
+      <c r="CL42">
         <v>0.1345972</v>
       </c>
       <c r="CU42" t="s">
@@ -3656,12 +3676,14 @@
       <c r="CV42">
         <v>10</v>
       </c>
-      <c r="CW42" s="11">
+      <c r="CW42">
         <v>0.96337409022310405</v>
       </c>
-      <c r="CX42" s="11"/>
-    </row>
-    <row r="43" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY42" s="11">
+        <v>0.75704580842886304</v>
+      </c>
+    </row>
+    <row r="43" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -3755,7 +3777,7 @@
       <c r="CK43">
         <v>0.69463728000000002</v>
       </c>
-      <c r="CL43" s="11">
+      <c r="CL43">
         <v>0.29181047999999998</v>
       </c>
       <c r="CU43" t="s">
@@ -3764,12 +3786,14 @@
       <c r="CV43">
         <v>11</v>
       </c>
-      <c r="CW43" s="11">
+      <c r="CW43">
         <v>0.30057450818491099</v>
       </c>
-      <c r="CX43" s="11"/>
-    </row>
-    <row r="44" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY43" s="11">
+        <v>0.180260463318169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -3863,7 +3887,7 @@
       <c r="CK44">
         <v>0.58370084</v>
       </c>
-      <c r="CL44" s="11">
+      <c r="CL44">
         <v>0.18548338</v>
       </c>
       <c r="CU44" t="s">
@@ -3872,12 +3896,14 @@
       <c r="CV44">
         <v>12</v>
       </c>
-      <c r="CW44" s="11">
+      <c r="CW44">
         <v>0.41817241380633002</v>
       </c>
-      <c r="CX44" s="11"/>
-    </row>
-    <row r="45" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY44" s="11">
+        <v>8.6279652232353204E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -3971,7 +3997,7 @@
       <c r="CK45">
         <v>0.91649906000000003</v>
       </c>
-      <c r="CL45" s="11">
+      <c r="CL45">
         <v>0.38815854</v>
       </c>
       <c r="CU45" t="s">
@@ -3980,12 +4006,14 @@
       <c r="CV45">
         <v>13</v>
       </c>
-      <c r="CW45" s="11">
+      <c r="CW45">
         <v>0.21760228250336799</v>
       </c>
-      <c r="CX45" s="11"/>
-    </row>
-    <row r="46" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY45" s="11">
+        <v>0.82051775619679601</v>
+      </c>
+    </row>
+    <row r="46" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -4079,7 +4107,7 @@
       <c r="CK46">
         <v>0.474657</v>
       </c>
-      <c r="CL46" s="11">
+      <c r="CL46">
         <v>0.27825873000000001</v>
       </c>
       <c r="CU46" t="s">
@@ -4088,12 +4116,14 @@
       <c r="CV46">
         <v>14</v>
       </c>
-      <c r="CW46" s="11">
+      <c r="CW46">
         <v>5.2087530798276001E-2</v>
       </c>
-      <c r="CX46" s="11"/>
-    </row>
-    <row r="47" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY46" s="11">
+        <v>0.35058503484102499</v>
+      </c>
+    </row>
+    <row r="47" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -4187,7 +4217,7 @@
       <c r="CK47">
         <v>0.67174752999999998</v>
       </c>
-      <c r="CL47" s="11">
+      <c r="CL47">
         <v>0.83269857999999997</v>
       </c>
       <c r="CU47" t="s">
@@ -4196,12 +4226,14 @@
       <c r="CV47">
         <v>15</v>
       </c>
-      <c r="CW47" s="11">
+      <c r="CW47">
         <v>0.18864788546957101</v>
       </c>
-      <c r="CX47" s="11"/>
-    </row>
-    <row r="48" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY47" s="11">
+        <v>9.5110296393490099E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -4295,7 +4327,7 @@
       <c r="CK48">
         <v>0.16183945</v>
       </c>
-      <c r="CL48" s="11">
+      <c r="CL48">
         <v>0.61753035999999994</v>
       </c>
       <c r="CU48" t="s">
@@ -4304,12 +4336,14 @@
       <c r="CV48">
         <v>16</v>
       </c>
-      <c r="CW48" s="11">
+      <c r="CW48">
         <v>0.33605977672704401</v>
       </c>
-      <c r="CX48" s="11"/>
-    </row>
-    <row r="49" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY48" s="11">
+        <v>0.409505576604415</v>
+      </c>
+    </row>
+    <row r="49" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -4403,7 +4437,7 @@
       <c r="CK49">
         <v>0.98521992000000003</v>
       </c>
-      <c r="CL49" s="11">
+      <c r="CL49">
         <v>6.9050200000000006E-2</v>
       </c>
       <c r="CU49" t="s">
@@ -4412,12 +4446,14 @@
       <c r="CV49">
         <v>17</v>
       </c>
-      <c r="CW49" s="11">
+      <c r="CW49">
         <v>6.5679907066020907E-2</v>
       </c>
-      <c r="CX49" s="11"/>
-    </row>
-    <row r="50" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY49" s="11">
+        <v>0.99840300945794302</v>
+      </c>
+    </row>
+    <row r="50" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>17</v>
       </c>
@@ -4511,7 +4547,7 @@
       <c r="CK50">
         <v>0.43340778000000002</v>
       </c>
-      <c r="CL50" s="11">
+      <c r="CL50">
         <v>0.25331931000000002</v>
       </c>
       <c r="CU50" t="s">
@@ -4520,12 +4556,14 @@
       <c r="CV50">
         <v>18</v>
       </c>
-      <c r="CW50" s="11">
+      <c r="CW50">
         <v>0.17470011204973901</v>
       </c>
-      <c r="CX50" s="11"/>
-    </row>
-    <row r="51" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY50" s="11">
+        <v>0.88979799954606797</v>
+      </c>
+    </row>
+    <row r="51" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -4619,7 +4657,7 @@
       <c r="CK51">
         <v>0.56122326</v>
       </c>
-      <c r="CL51" s="11">
+      <c r="CL51">
         <v>0.91811350999999997</v>
       </c>
       <c r="CU51" t="s">
@@ -4628,12 +4666,14 @@
       <c r="CV51">
         <v>19</v>
       </c>
-      <c r="CW51" s="11">
+      <c r="CW51">
         <v>0.50852101612879896</v>
       </c>
-      <c r="CX51" s="11"/>
-    </row>
-    <row r="52" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY51" s="11">
+        <v>8.8274050199137297E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -4727,7 +4767,7 @@
       <c r="CK52">
         <v>0.72634069000000001</v>
       </c>
-      <c r="CL52" s="11">
+      <c r="CL52">
         <v>0.57604443000000005</v>
       </c>
       <c r="CU52" t="s">
@@ -4736,12 +4776,14 @@
       <c r="CV52">
         <v>20</v>
       </c>
-      <c r="CW52" s="11">
+      <c r="CW52">
         <v>0.21394113718953101</v>
       </c>
-      <c r="CX52" s="11"/>
-    </row>
-    <row r="53" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY52" s="11">
+        <v>0.35702305540287399</v>
+      </c>
+    </row>
+    <row r="53" spans="1:103" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -4835,7 +4877,7 @@
       <c r="CK53">
         <v>0.92028133000000001</v>
       </c>
-      <c r="CL53" s="11">
+      <c r="CL53">
         <v>0.15545563000000001</v>
       </c>
       <c r="CU53" t="s">
@@ -4844,12 +4886,14 @@
       <c r="CV53">
         <v>21</v>
       </c>
-      <c r="CW53" s="11">
+      <c r="CW53">
         <v>0.73894155683004903</v>
       </c>
-      <c r="CX53" s="11"/>
-    </row>
-    <row r="54" spans="1:102" x14ac:dyDescent="0.25">
+      <c r="CY53" s="11">
+        <v>0.58802578819175599</v>
+      </c>
+    </row>
+    <row r="54" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK54" t="s">
         <v>55</v>
       </c>
@@ -4879,7 +4923,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK55" t="s">
         <v>54</v>
       </c>
@@ -4903,7 +4947,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK56" t="s">
         <v>53</v>
       </c>
@@ -4927,7 +4971,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK57" t="s">
         <v>52</v>
       </c>
@@ -4955,7 +4999,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="58" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK58" t="s">
         <v>58</v>
       </c>
@@ -4983,7 +5027,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="59" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK59" t="s">
         <v>51</v>
       </c>
@@ -5003,7 +5047,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="60" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:103" x14ac:dyDescent="0.25">
       <c r="AK60" t="s">
         <v>50</v>
       </c>
@@ -5023,79 +5067,79 @@
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:103" x14ac:dyDescent="0.25">
       <c r="Z63" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="64" spans="1:102" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="64" spans="1:103" x14ac:dyDescent="0.25">
       <c r="Z64" t="str" cm="1">
         <f t="array" ref="Z64:AT64">_xlfn.TEXTSPLIT(Z63,", ")</f>
-        <v>0.4091753041621535</v>
+        <v>0.4679608226343523</v>
       </c>
       <c r="AA64" t="str">
-        <v>0.526987531425831</v>
+        <v>0.9362630083244707</v>
       </c>
       <c r="AB64" t="str">
-        <v>0.07765675894938162</v>
+        <v>0.045734449308683464</v>
       </c>
       <c r="AC64" t="str">
-        <v>0.004964104866896055</v>
+        <v>0.12002048293538281</v>
       </c>
       <c r="AD64" t="str">
-        <v>0.6199393341507159</v>
+        <v>0.9753029321700649</v>
       </c>
       <c r="AE64" t="str">
-        <v>0.7247614063773686</v>
+        <v>0.9216730696463928</v>
       </c>
       <c r="AF64" t="str">
-        <v>0.45860226419395134</v>
+        <v>0.2557964891936836</v>
       </c>
       <c r="AG64" t="str">
-        <v>0.15632117815261173</v>
+        <v>0.027180268139501307</v>
       </c>
       <c r="AH64" t="str">
-        <v>0.40243406150630634</v>
+        <v>0.9210008983160494</v>
       </c>
       <c r="AI64" t="str">
-        <v>0.963374090223104</v>
+        <v>0.7570458084288632</v>
       </c>
       <c r="AJ64" t="str">
-        <v>0.3005745081849112</v>
+        <v>0.18026046331816964</v>
       </c>
       <c r="AK64" t="str">
-        <v>0.4181724138063309</v>
+        <v>0.08627965223235323</v>
       </c>
       <c r="AL64" t="str">
-        <v>0.217602282503368</v>
+        <v>0.820517756196796</v>
       </c>
       <c r="AM64" t="str">
-        <v>0.05208753079827609</v>
+        <v>0.3505850348410258</v>
       </c>
       <c r="AN64" t="str">
-        <v>0.18864788546957187</v>
+        <v>0.09511029639349017</v>
       </c>
       <c r="AO64" t="str">
-        <v>0.3360597767270444</v>
+        <v>0.4095055766044159</v>
       </c>
       <c r="AP64" t="str">
-        <v>0.06567990706602098</v>
+        <v>0.9984030094579434</v>
       </c>
       <c r="AQ64" t="str">
-        <v>0.1747001120497397</v>
+        <v>0.8897979995460684</v>
       </c>
       <c r="AR64" t="str">
-        <v>0.5085210161287994</v>
+        <v>0.08827405019913738</v>
       </c>
       <c r="AS64" t="str">
-        <v>0.21394113718953117</v>
+        <v>0.3570230554028749</v>
       </c>
       <c r="AT64" t="str">
-        <v>0.7389415568300491</v>
+        <v>0.5880257881917569</v>
       </c>
     </row>
     <row r="65" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X65" s="10">
+      <c r="X65" s="3">
         <v>0.33831719711374802</v>
       </c>
       <c r="Y65">
@@ -5103,18 +5147,18 @@
       </c>
       <c r="Z65" s="3" t="str" cm="1">
         <f t="array" ref="Z65:Z85">TRANSPOSE(_xlfn.ANCHORARRAY(Z64))</f>
-        <v>0.4091753041621535</v>
+        <v>0.4679608226343523</v>
       </c>
     </row>
     <row r="66" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X66" s="9">
+      <c r="X66" s="2">
         <v>0.93466713178917704</v>
       </c>
       <c r="Y66">
         <v>2</v>
       </c>
       <c r="Z66" s="2" t="str">
-        <v>0.526987531425831</v>
+        <v>0.9362630083244707</v>
       </c>
       <c r="AZ66" s="3">
         <v>0.33831719711374802</v>
@@ -5136,18 +5180,18 @@
       </c>
       <c r="BH66" t="str">
         <f>_xlfn.TEXTJOIN("#",TRUE,BF67:BF87)</f>
-        <v>0.409175#0.526988#0.077657#0.004964#0.619939#0.724761#0.458602#0.156321#0.402434#0.963374#0.300575#0.418172#0.217602#0.052088#0.188648#0.33606#0.06568#0.1747#0.508521#0.213941#0.738942</v>
+        <v>0.467960822634352#0.93626300832447#0.0457344493086834#0.120020482935382#0.975302932170064#0.921673069646392#0.255796489193683#0.0271802681395013#0.921000898316049#0.757045808428863#0.180260463318169#0.0862796522323532#0.820517756196796#0.350585034841025#0.0951102963934901#0.409505576604415#0.998403009457943#0.889797999546068#0.0882740501991373#0.357023055402874#0.588025788191756</v>
       </c>
     </row>
     <row r="67" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X67" s="10">
+      <c r="X67" s="3">
         <v>9.3176192652155904E-2</v>
       </c>
       <c r="Y67">
         <v>3</v>
       </c>
       <c r="Z67" s="3" t="str">
-        <v>0.07765675894938162</v>
+        <v>0.045734449308683464</v>
       </c>
       <c r="AZ67" s="2">
         <v>0.93466713178917704</v>
@@ -5156,29 +5200,29 @@
         <v>34</v>
       </c>
       <c r="BB67">
-        <f t="shared" ref="BB67:BB86" si="1">AZ67-BA67</f>
+        <f t="shared" ref="BB67:BB86" si="3">AZ67-BA67</f>
         <v>-6.5332868210822959E-2</v>
       </c>
       <c r="BC67">
         <v>6.5332868210822959E-2</v>
       </c>
-      <c r="BF67" s="12">
-        <v>0.40917500000000001</v>
+      <c r="BF67" s="8">
+        <v>0.46796082263435201</v>
       </c>
       <c r="BH67" t="str">
         <f>_xlfn.REGEXREPLACE(BH66," ","")</f>
-        <v>0.409175#0.526988#0.077657#0.004964#0.619939#0.724761#0.458602#0.156321#0.402434#0.963374#0.300575#0.418172#0.217602#0.052088#0.188648#0.33606#0.06568#0.1747#0.508521#0.213941#0.738942</v>
+        <v>0.467960822634352#0.93626300832447#0.0457344493086834#0.120020482935382#0.975302932170064#0.921673069646392#0.255796489193683#0.0271802681395013#0.921000898316049#0.757045808428863#0.180260463318169#0.0862796522323532#0.820517756196796#0.350585034841025#0.0951102963934901#0.409505576604415#0.998403009457943#0.889797999546068#0.0882740501991373#0.357023055402874#0.588025788191756</v>
       </c>
     </row>
     <row r="68" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X68" s="9">
+      <c r="X68" s="2">
         <v>0</v>
       </c>
       <c r="Y68">
         <v>4</v>
       </c>
       <c r="Z68" s="2" t="str">
-        <v>0.004964104866896055</v>
+        <v>0.12002048293538281</v>
       </c>
       <c r="AB68" t="str">
         <f>_xlfn.TEXTJOIN("#",FALSE,X65:X85)</f>
@@ -5191,28 +5235,28 @@
         <v>35</v>
       </c>
       <c r="BB68">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>9.3176192652155904E-2</v>
       </c>
       <c r="BC68">
         <v>9.3176192652155904E-2</v>
       </c>
-      <c r="BF68" s="13">
-        <v>0.52698800000000001</v>
+      <c r="BF68" s="9">
+        <v>0.93626300832446996</v>
       </c>
       <c r="BH68" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X69" s="10">
+      <c r="X69" s="3">
         <v>0.75109902463000799</v>
       </c>
       <c r="Y69">
         <v>5</v>
       </c>
       <c r="Z69" s="3" t="str">
-        <v>0.6199393341507159</v>
+        <v>0.9753029321700649</v>
       </c>
       <c r="AZ69" s="2">
         <v>0</v>
@@ -5221,28 +5265,28 @@
         <v>35</v>
       </c>
       <c r="BB69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="BC69">
         <v>0</v>
       </c>
-      <c r="BF69" s="12">
-        <v>7.7657000000000004E-2</v>
+      <c r="BF69" s="8">
+        <v>4.5734449308683402E-2</v>
       </c>
       <c r="BH69" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="70" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X70" s="9">
+      <c r="X70" s="2">
         <v>1</v>
       </c>
       <c r="Y70">
         <v>6</v>
       </c>
       <c r="Z70" s="2" t="str">
-        <v>0.7247614063773686</v>
+        <v>0.9216730696463928</v>
       </c>
       <c r="AB70" t="s">
         <v>115</v>
@@ -5254,28 +5298,28 @@
         <v>34</v>
       </c>
       <c r="BB70">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.24890097536999201</v>
       </c>
       <c r="BC70">
         <v>0.24890097536999201</v>
       </c>
-      <c r="BF70" s="13">
-        <v>4.9639999999999997E-3</v>
+      <c r="BF70" s="9">
+        <v>0.12002048293538201</v>
       </c>
       <c r="BH70" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="71" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X71" s="10">
+      <c r="X71" s="3">
         <v>0.96184788633787499</v>
       </c>
       <c r="Y71">
         <v>7</v>
       </c>
       <c r="Z71" s="3" t="str">
-        <v>0.45860226419395134</v>
+        <v>0.2557964891936836</v>
       </c>
       <c r="AB71" t="s">
         <v>114</v>
@@ -5287,25 +5331,25 @@
         <v>34</v>
       </c>
       <c r="BB71">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="BC71">
         <v>0</v>
       </c>
-      <c r="BF71" s="12">
-        <v>0.61993900000000002</v>
+      <c r="BF71" s="8">
+        <v>0.97530293217006403</v>
       </c>
     </row>
     <row r="72" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X72" s="9">
+      <c r="X72" s="2">
         <v>0</v>
       </c>
       <c r="Y72">
         <v>8</v>
       </c>
       <c r="Z72" s="2" t="str">
-        <v>0.15632117815261173</v>
+        <v>0.027180268139501307</v>
       </c>
       <c r="AB72" t="s">
         <v>110</v>
@@ -5317,25 +5361,25 @@
         <v>34</v>
       </c>
       <c r="BB72">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-3.8152113662125009E-2</v>
       </c>
       <c r="BC72">
         <v>3.8152113662125009E-2</v>
       </c>
-      <c r="BF72" s="13">
-        <v>0.72476099999999999</v>
+      <c r="BF72" s="9">
+        <v>0.92167306964639195</v>
       </c>
     </row>
     <row r="73" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X73" s="10">
+      <c r="X73" s="3">
         <v>1</v>
       </c>
       <c r="Y73">
         <v>9</v>
       </c>
       <c r="Z73" s="3" t="str">
-        <v>0.40243406150630634</v>
+        <v>0.9210008983160494</v>
       </c>
       <c r="AZ73" s="2">
         <v>0</v>
@@ -5344,28 +5388,28 @@
         <v>35</v>
       </c>
       <c r="BB73">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="BC73">
         <v>0</v>
       </c>
-      <c r="BF73" s="12">
-        <v>0.45860200000000001</v>
+      <c r="BF73" s="8">
+        <v>0.25579648919368297</v>
       </c>
       <c r="BH73" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="74" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X74" s="9">
+      <c r="X74" s="2">
         <v>0.55293794800527796</v>
       </c>
       <c r="Y74">
         <v>10</v>
       </c>
       <c r="Z74" s="2" t="str">
-        <v>0.963374090223104</v>
+        <v>0.7570458084288632</v>
       </c>
       <c r="AZ74" s="3">
         <v>1</v>
@@ -5374,25 +5418,25 @@
         <v>36</v>
       </c>
       <c r="BB74">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.13852660842636</v>
       </c>
       <c r="BC74">
         <v>0.13852660842636</v>
       </c>
-      <c r="BF74" s="13">
-        <v>0.15632099999999999</v>
+      <c r="BF74" s="9">
+        <v>2.71802681395013E-2</v>
       </c>
     </row>
     <row r="75" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X75" s="10">
+      <c r="X75" s="3">
         <v>0.59671345821399002</v>
       </c>
       <c r="Y75">
         <v>11</v>
       </c>
       <c r="Z75" s="3" t="str">
-        <v>0.3005745081849112</v>
+        <v>0.18026046331816964</v>
       </c>
       <c r="AZ75" s="2">
         <v>0.55293794800527796</v>
@@ -5401,25 +5445,25 @@
         <v>34</v>
       </c>
       <c r="BB75">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.44706205199472204</v>
       </c>
       <c r="BC75">
         <v>0.44706205199472204</v>
       </c>
-      <c r="BF75" s="12">
-        <v>0.40243400000000001</v>
+      <c r="BF75" s="8">
+        <v>0.92100089831604903</v>
       </c>
     </row>
     <row r="76" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X76" s="9">
+      <c r="X76" s="2">
         <v>0</v>
       </c>
       <c r="Y76">
         <v>12</v>
       </c>
       <c r="Z76" s="2" t="str">
-        <v>0.4181724138063309</v>
+        <v>0.08627965223235323</v>
       </c>
       <c r="AZ76" s="3">
         <v>0.59671345821399002</v>
@@ -5428,25 +5472,25 @@
         <v>37</v>
       </c>
       <c r="BB76">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.3686848516020014E-2</v>
       </c>
       <c r="BC76">
         <v>5.3686848516020014E-2</v>
       </c>
-      <c r="BF76" s="13">
-        <v>0.96337399999999995</v>
+      <c r="BF76" s="9">
+        <v>0.75704580842886304</v>
       </c>
     </row>
     <row r="77" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X77" s="10">
+      <c r="X77" s="3">
         <v>1</v>
       </c>
       <c r="Y77">
         <v>13</v>
       </c>
       <c r="Z77" s="3" t="str">
-        <v>0.217602282503368</v>
+        <v>0.820517756196796</v>
       </c>
       <c r="AZ77" s="2">
         <v>0</v>
@@ -5455,25 +5499,25 @@
         <v>34</v>
       </c>
       <c r="BB77">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
       <c r="BC77">
         <v>1</v>
       </c>
-      <c r="BF77" s="12">
-        <v>0.30057499999999998</v>
+      <c r="BF77" s="8">
+        <v>0.180260463318169</v>
       </c>
     </row>
     <row r="78" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X78" s="9">
+      <c r="X78" s="2">
         <v>0</v>
       </c>
       <c r="Y78">
         <v>14</v>
       </c>
       <c r="Z78" s="2" t="str">
-        <v>0.05208753079827609</v>
+        <v>0.3505850348410258</v>
       </c>
       <c r="AZ78" s="3">
         <v>1</v>
@@ -5482,25 +5526,25 @@
         <v>35</v>
       </c>
       <c r="BB78">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="BC78">
         <v>1</v>
       </c>
-      <c r="BF78" s="13">
-        <v>0.41817199999999999</v>
+      <c r="BF78" s="9">
+        <v>8.6279652232353204E-2</v>
       </c>
     </row>
     <row r="79" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X79" s="10">
+      <c r="X79" s="3">
         <v>0</v>
       </c>
       <c r="Y79">
         <v>15</v>
       </c>
       <c r="Z79" s="3" t="str">
-        <v>0.18864788546957187</v>
+        <v>0.09511029639349017</v>
       </c>
       <c r="AZ79" s="2">
         <v>0</v>
@@ -5509,25 +5553,25 @@
         <v>38</v>
       </c>
       <c r="BB79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.17621606443353</v>
       </c>
       <c r="BC79">
         <v>0.17621606443353</v>
       </c>
-      <c r="BF79" s="12">
-        <v>0.21760199999999999</v>
+      <c r="BF79" s="8">
+        <v>0.82051775619679601</v>
       </c>
     </row>
     <row r="80" spans="24:60" x14ac:dyDescent="0.25">
-      <c r="X80" s="9">
+      <c r="X80" s="2">
         <v>1</v>
       </c>
       <c r="Y80">
         <v>16</v>
       </c>
       <c r="Z80" s="2" t="str">
-        <v>0.3360597767270444</v>
+        <v>0.4095055766044159</v>
       </c>
       <c r="AZ80" s="3">
         <v>0</v>
@@ -5536,25 +5580,25 @@
         <v>34</v>
       </c>
       <c r="BB80">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
       <c r="BC80">
         <v>1</v>
       </c>
-      <c r="BF80" s="13">
-        <v>5.2088000000000002E-2</v>
+      <c r="BF80" s="9">
+        <v>0.35058503484102499</v>
       </c>
     </row>
     <row r="81" spans="24:58" x14ac:dyDescent="0.25">
-      <c r="X81" s="10">
+      <c r="X81" s="3">
         <v>0</v>
       </c>
       <c r="Y81">
         <v>17</v>
       </c>
       <c r="Z81" s="3" t="str">
-        <v>0.06567990706602098</v>
+        <v>0.9984030094579434</v>
       </c>
       <c r="AZ81" s="2">
         <v>1</v>
@@ -5563,25 +5607,25 @@
         <v>39</v>
       </c>
       <c r="BB81">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.58957907790050801</v>
       </c>
       <c r="BC81">
         <v>0.58957907790050801</v>
       </c>
-      <c r="BF81" s="12">
-        <v>0.18864800000000001</v>
+      <c r="BF81" s="8">
+        <v>9.5110296393490099E-2</v>
       </c>
     </row>
     <row r="82" spans="24:58" x14ac:dyDescent="0.25">
-      <c r="X82" s="9">
+      <c r="X82" s="2">
         <v>2.1401265694797498E-3</v>
       </c>
       <c r="Y82">
         <v>18</v>
       </c>
       <c r="Z82" s="2" t="str">
-        <v>0.1747001120497397</v>
+        <v>0.8897979995460684</v>
       </c>
       <c r="AZ82" s="3">
         <v>0</v>
@@ -5590,25 +5634,25 @@
         <v>40</v>
       </c>
       <c r="BB82">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.93748321022143899</v>
       </c>
       <c r="BC82">
         <v>0.93748321022143899</v>
       </c>
-      <c r="BF82" s="13">
-        <v>0.33606000000000003</v>
+      <c r="BF82" s="9">
+        <v>0.409505576604415</v>
       </c>
     </row>
     <row r="83" spans="24:58" x14ac:dyDescent="0.25">
-      <c r="X83" s="10">
+      <c r="X83" s="3">
         <v>0.37166843346534201</v>
       </c>
       <c r="Y83">
         <v>19</v>
       </c>
       <c r="Z83" s="3" t="str">
-        <v>0.5085210161287994</v>
+        <v>0.08827405019913738</v>
       </c>
       <c r="AZ83" s="2">
         <v>2.1401265694797498E-3</v>
@@ -5617,25 +5661,25 @@
         <v>34</v>
       </c>
       <c r="BB83">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.99785987343052029</v>
       </c>
       <c r="BC83">
         <v>0.99785987343052029</v>
       </c>
-      <c r="BF83" s="12">
-        <v>6.5680000000000002E-2</v>
+      <c r="BF83" s="8">
+        <v>0.99840300945794302</v>
       </c>
     </row>
     <row r="84" spans="24:58" x14ac:dyDescent="0.25">
-      <c r="X84" s="9">
+      <c r="X84" s="2">
         <v>0.16946907320228299</v>
       </c>
       <c r="Y84">
         <v>20</v>
       </c>
       <c r="Z84" s="2" t="str">
-        <v>0.21394113718953117</v>
+        <v>0.3570230554028749</v>
       </c>
       <c r="AZ84" s="3">
         <v>0.37166843346534201</v>
@@ -5644,25 +5688,25 @@
         <v>41</v>
       </c>
       <c r="BB84">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7.8902838744676018E-2</v>
       </c>
       <c r="BC84">
         <v>7.8902838744676018E-2</v>
       </c>
-      <c r="BF84" s="13">
-        <v>0.17469999999999999</v>
+      <c r="BF84" s="9">
+        <v>0.88979799954606797</v>
       </c>
     </row>
     <row r="85" spans="24:58" x14ac:dyDescent="0.25">
-      <c r="X85" s="10">
+      <c r="X85" s="3">
         <v>0</v>
       </c>
       <c r="Y85">
         <v>21</v>
       </c>
       <c r="Z85" s="3" t="str">
-        <v>0.7389415568300491</v>
+        <v>0.5880257881917569</v>
       </c>
       <c r="AZ85" s="2">
         <v>0.16946907320228299</v>
@@ -5671,14 +5715,14 @@
         <v>42</v>
       </c>
       <c r="BB85">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.15121010424644088</v>
       </c>
       <c r="BC85">
         <v>0.15121010424644088</v>
       </c>
-      <c r="BF85" s="12">
-        <v>0.508521</v>
+      <c r="BF85" s="8">
+        <v>8.8274050199137297E-2</v>
       </c>
     </row>
     <row r="86" spans="24:58" x14ac:dyDescent="0.25">
@@ -5693,14 +5737,14 @@
         <v>43</v>
       </c>
       <c r="BB86">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-0.28901297450699598</v>
       </c>
       <c r="BC86">
         <v>0.28901297450699598</v>
       </c>
-      <c r="BF86" s="13">
-        <v>0.21394099999999999</v>
+      <c r="BF86" s="9">
+        <v>0.35702305540287399</v>
       </c>
     </row>
     <row r="87" spans="24:58" x14ac:dyDescent="0.25">
@@ -5711,8 +5755,8 @@
       <c r="BA87" t="s">
         <v>44</v>
       </c>
-      <c r="BF87" s="12">
-        <v>0.73894199999999999</v>
+      <c r="BF87" s="8">
+        <v>0.58802578819175599</v>
       </c>
     </row>
     <row r="88" spans="24:58" x14ac:dyDescent="0.25">
@@ -5782,19 +5826,19 @@
       </c>
       <c r="AI91" s="5">
         <f ca="1">RAND()*0.1-0.05</f>
-        <v>1.1916031306460885E-2</v>
+        <v>3.9746935981963147E-2</v>
       </c>
       <c r="AJ91" s="5">
         <f ca="1">MIN(MAX(AH91+AI91,0),1)</f>
-        <v>1.1916031306460885E-2</v>
+        <v>3.9746935981963147E-2</v>
       </c>
       <c r="AK91" s="5">
-        <f t="shared" ref="AK91:AK111" ca="1" si="2">RAND()*0.1-0.05</f>
-        <v>2.0428177172587353E-2</v>
+        <f t="shared" ref="AK91:AK111" ca="1" si="4">RAND()*0.1-0.05</f>
+        <v>-3.2143402752549066E-2</v>
       </c>
       <c r="AL91" s="5">
         <f ca="1">MIN(MAX(AJ91+AK91,0),1)</f>
-        <v>3.2344208479048238E-2</v>
+        <v>7.6035332294140806E-3</v>
       </c>
       <c r="BA91" t="s">
         <v>47</v>
@@ -5812,20 +5856,20 @@
         <v>0.838073450710207</v>
       </c>
       <c r="AI92" s="5">
-        <f t="shared" ref="AI92:AI111" ca="1" si="3">RAND()*0.1-0.05</f>
-        <v>4.6706814426305185E-2</v>
+        <f t="shared" ref="AI92:AI111" ca="1" si="5">RAND()*0.1-0.05</f>
+        <v>-9.4463885445216084E-3</v>
       </c>
       <c r="AJ92" s="5">
-        <f t="shared" ref="AJ92:AJ111" ca="1" si="4">MIN(MAX(AH92+AI92,0),1)</f>
-        <v>0.8847802651365122</v>
+        <f t="shared" ref="AJ92:AJ111" ca="1" si="6">MIN(MAX(AH92+AI92,0),1)</f>
+        <v>0.82862706216568538</v>
       </c>
       <c r="AK92" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-1.4234668444242017E-2</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>-1.3139185304644287E-2</v>
       </c>
       <c r="AL92" s="5">
-        <f t="shared" ref="AL92:AL111" ca="1" si="5">MIN(MAX(AJ92+AK92,0),1)</f>
-        <v>0.87054559669227016</v>
+        <f t="shared" ref="AL92:AL111" ca="1" si="7">MIN(MAX(AJ92+AK92,0),1)</f>
+        <v>0.81548787686104107</v>
       </c>
       <c r="BA92" t="s">
         <v>48</v>
@@ -5842,20 +5886,20 @@
         <v>0.36941805210713202</v>
       </c>
       <c r="AI93" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>3.2019769218140884E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>8.7859707949001567E-3</v>
       </c>
       <c r="AJ93" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.3782040229020322</v>
+      </c>
+      <c r="AK93" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.40143782132527289</v>
-      </c>
-      <c r="AK93" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.3866307009600166E-2</v>
+        <v>-3.4207409626422991E-2</v>
       </c>
       <c r="AL93" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.3675715143156727</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.34399661327560921</v>
       </c>
       <c r="BA93" t="s">
         <v>34</v>
@@ -5872,20 +5916,20 @@
         <v>0.772175920311859</v>
       </c>
       <c r="AI94" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-4.2127407015037921E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>3.5692963106022269E-2</v>
       </c>
       <c r="AJ94" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.80786888341788132</v>
+      </c>
+      <c r="AK94" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.73004851329682108</v>
-      </c>
-      <c r="AK94" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>9.8416288978085201E-3</v>
+        <v>4.2304338618809487E-2</v>
       </c>
       <c r="AL94" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.73989014219462956</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.85017322203669077</v>
       </c>
     </row>
     <row r="95" spans="24:58" x14ac:dyDescent="0.25">
@@ -5899,20 +5943,20 @@
         <v>0.61234593074099897</v>
       </c>
       <c r="AI95" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-3.0927995758098473E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-3.4923447863014372E-2</v>
       </c>
       <c r="AJ95" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.57742248287798459</v>
+      </c>
+      <c r="AK95" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.58141793498290051</v>
-      </c>
-      <c r="AK95" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>8.8959608536855195E-4</v>
+        <v>4.36486956721268E-3</v>
       </c>
       <c r="AL95" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.58230753106826905</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.5817873524451973</v>
       </c>
     </row>
     <row r="96" spans="24:58" x14ac:dyDescent="0.25">
@@ -5926,20 +5970,20 @@
         <v>0</v>
       </c>
       <c r="AI96" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>2.9233313097612484E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>7.0298942926227612E-3</v>
       </c>
       <c r="AJ96" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>7.0298942926227612E-3</v>
+      </c>
+      <c r="AK96" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>2.9233313097612484E-2</v>
-      </c>
-      <c r="AK96" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.852895702953002E-2</v>
+        <v>2.2569668822687988E-2</v>
       </c>
       <c r="AL96" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>2.9599563115310749E-2</v>
       </c>
     </row>
     <row r="97" spans="25:38" x14ac:dyDescent="0.25">
@@ -5953,20 +5997,20 @@
         <v>1</v>
       </c>
       <c r="AI97" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>3.810932319159295E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-1.0682744863139637E-2</v>
       </c>
       <c r="AJ97" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.98931725513686031</v>
+      </c>
+      <c r="AK97" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="AK97" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.2086140754052028E-2</v>
+        <v>3.7401897116818308E-2</v>
       </c>
       <c r="AL97" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.96791385924594797</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="25:38" x14ac:dyDescent="0.25">
@@ -5980,20 +6024,20 @@
         <v>0.27929680791088402</v>
       </c>
       <c r="AI98" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-4.3221285094681067E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>4.8984518852293255E-2</v>
       </c>
       <c r="AJ98" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.32828132676317728</v>
+      </c>
+      <c r="AK98" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.23607552281620295</v>
-      </c>
-      <c r="AK98" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>1.3866523899752098E-2</v>
+        <v>-2.2352860448700596E-2</v>
       </c>
       <c r="AL98" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.24994204671595505</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.30592846631447668</v>
       </c>
     </row>
     <row r="99" spans="25:38" x14ac:dyDescent="0.25">
@@ -6007,20 +6051,20 @@
         <v>1</v>
       </c>
       <c r="AI99" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-3.4398954097546224E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>3.6033190368486942E-2</v>
       </c>
       <c r="AJ99" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK99" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.96560104590245377</v>
-      </c>
-      <c r="AK99" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>2.1043001645684262E-2</v>
+        <v>3.6417212825623255E-2</v>
       </c>
       <c r="AL99" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.98664404754813806</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="25:38" x14ac:dyDescent="0.25">
@@ -6034,20 +6078,20 @@
         <v>3.9908815338230499E-2</v>
       </c>
       <c r="AI100" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>1.7565624915193145E-4</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-1.6206031857341131E-2</v>
       </c>
       <c r="AJ100" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>2.3702783480889368E-2</v>
+      </c>
+      <c r="AK100" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>4.0084471587382431E-2</v>
-      </c>
-      <c r="AK100" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>2.2598677687330065E-2</v>
+        <v>-7.9800786505243165E-3</v>
       </c>
       <c r="AL100" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>6.2683149274712496E-2</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>1.5722704830365052E-2</v>
       </c>
     </row>
     <row r="101" spans="25:38" x14ac:dyDescent="0.25">
@@ -6061,20 +6105,20 @@
         <v>0.93716941113188901</v>
       </c>
       <c r="AI101" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>2.1515469868834985E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-5.9632346753396015E-3</v>
       </c>
       <c r="AJ101" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.93120617645654935</v>
+      </c>
+      <c r="AK101" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.95868488100072402</v>
-      </c>
-      <c r="AK101" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>3.3634848093355499E-3</v>
+        <v>-1.1342451923918098E-2</v>
       </c>
       <c r="AL101" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.96204836581005959</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.91986372453263121</v>
       </c>
     </row>
     <row r="102" spans="25:38" x14ac:dyDescent="0.25">
@@ -6088,20 +6132,20 @@
         <v>1</v>
       </c>
       <c r="AI102" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>2.8170111367688738E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1.5744485397105157E-2</v>
       </c>
       <c r="AJ102" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK102" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="AK102" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>2.1134994966465412E-2</v>
+        <v>-2.4164000424158463E-2</v>
       </c>
       <c r="AL102" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.97583599957584155</v>
       </c>
     </row>
     <row r="103" spans="25:38" x14ac:dyDescent="0.25">
@@ -6115,20 +6159,20 @@
         <v>0.62226011233405598</v>
       </c>
       <c r="AI103" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>1.8134462873401341E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>3.5766927373168805E-3</v>
       </c>
       <c r="AJ103" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.62583680507137285</v>
+      </c>
+      <c r="AK103" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.64039457520745735</v>
-      </c>
-      <c r="AK103" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>4.0492971239076456E-2</v>
+        <v>-4.3362296152969042E-2</v>
       </c>
       <c r="AL103" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.68088754644653382</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.5824745089184038</v>
       </c>
     </row>
     <row r="104" spans="25:38" x14ac:dyDescent="0.25">
@@ -6142,20 +6186,20 @@
         <v>0</v>
       </c>
       <c r="AI104" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>4.0063381798908962E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-1.6669180228889767E-2</v>
       </c>
       <c r="AJ104" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AK104" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>4.0063381798908962E-2</v>
-      </c>
-      <c r="AK104" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-2.3329342130141054E-2</v>
+        <v>2.7119814094726899E-2</v>
       </c>
       <c r="AL104" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>1.6734039668767908E-2</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>2.7119814094726899E-2</v>
       </c>
     </row>
     <row r="105" spans="25:38" x14ac:dyDescent="0.25">
@@ -6169,20 +6213,20 @@
         <v>0.55344351954543602</v>
       </c>
       <c r="AI105" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-3.4416935114258529E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-1.7959165721740299E-2</v>
       </c>
       <c r="AJ105" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.53548435382369575</v>
+      </c>
+      <c r="AK105" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.51902658443117744</v>
-      </c>
-      <c r="AK105" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.1640846762434151E-2</v>
+        <v>-1.762601405166183E-2</v>
       </c>
       <c r="AL105" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.48738573766874327</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.51785833977203388</v>
       </c>
     </row>
     <row r="106" spans="25:38" x14ac:dyDescent="0.25">
@@ -6196,20 +6240,20 @@
         <v>0.78854921023547897</v>
       </c>
       <c r="AI106" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>3.7175583616828406E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-4.7334515856491982E-2</v>
       </c>
       <c r="AJ106" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.74121469437898702</v>
+      </c>
+      <c r="AK106" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.82572479385230735</v>
-      </c>
-      <c r="AK106" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.1469344697524645E-2</v>
+        <v>3.7720003676931721E-3</v>
       </c>
       <c r="AL106" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.79425544915478274</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.74498669474668022</v>
       </c>
     </row>
     <row r="107" spans="25:38" x14ac:dyDescent="0.25">
@@ -6223,20 +6267,20 @@
         <v>0.34360099288912299</v>
       </c>
       <c r="AI107" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>3.2783217514491578E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>4.1343023896895648E-2</v>
       </c>
       <c r="AJ107" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.38494401678601864</v>
+      </c>
+      <c r="AK107" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.37638421040361458</v>
-      </c>
-      <c r="AK107" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-3.0852466495419839E-2</v>
+        <v>3.2776057786693624E-2</v>
       </c>
       <c r="AL107" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.34553174390819474</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.41772007457271226</v>
       </c>
     </row>
     <row r="108" spans="25:38" x14ac:dyDescent="0.25">
@@ -6250,20 +6294,20 @@
         <v>0</v>
       </c>
       <c r="AI108" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>3.3039256769751169E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1.8934843425303244E-2</v>
       </c>
       <c r="AJ108" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>1.8934843425303244E-2</v>
+      </c>
+      <c r="AK108" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>3.3039256769751169E-2</v>
-      </c>
-      <c r="AK108" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-2.3019134604962091E-2</v>
+        <v>1.7747025674528405E-2</v>
       </c>
       <c r="AL108" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>1.0020122164789078E-2</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>3.6681869099831649E-2</v>
       </c>
     </row>
     <row r="109" spans="25:38" x14ac:dyDescent="0.25">
@@ -6277,20 +6321,20 @@
         <v>0.34378680064676098</v>
       </c>
       <c r="AI109" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-3.2291137506626821E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>1.8040402232156333E-2</v>
       </c>
       <c r="AJ109" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.36182720287891734</v>
+      </c>
+      <c r="AK109" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.31149566314013416</v>
-      </c>
-      <c r="AK109" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>3.2039608658353536E-2</v>
+        <v>8.0784727460448402E-3</v>
       </c>
       <c r="AL109" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.3435352717984877</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.36990567562496218</v>
       </c>
     </row>
     <row r="110" spans="25:38" x14ac:dyDescent="0.25">
@@ -6304,20 +6348,20 @@
         <v>1</v>
       </c>
       <c r="AI110" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>-1.522874914713819E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>-5.5546200060767811E-3</v>
       </c>
       <c r="AJ110" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>0.99444537999392324</v>
+      </c>
+      <c r="AK110" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>0.98477125085286177</v>
-      </c>
-      <c r="AK110" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-6.2039574049288088E-3</v>
+        <v>2.4120672148275624E-2</v>
       </c>
       <c r="AL110" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.97856729344793292</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="25:38" x14ac:dyDescent="0.25">
@@ -6331,20 +6375,20 @@
         <v>1</v>
       </c>
       <c r="AI111" s="5">
-        <f t="shared" ca="1" si="3"/>
-        <v>1.623837575593072E-2</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>3.4013403868717471E-2</v>
       </c>
       <c r="AJ111" s="5">
+        <f t="shared" ca="1" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK111" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="AK111" s="5">
-        <f t="shared" ca="1" si="2"/>
-        <v>-4.8408167853834394E-2</v>
+        <v>-3.5869802513916485E-2</v>
       </c>
       <c r="AL111" s="5">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.95159183214616561</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>0.96413019748608353</v>
       </c>
     </row>
     <row r="112" spans="25:38" x14ac:dyDescent="0.25">
@@ -6495,201 +6539,202 @@
     <col min="76" max="76" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="77" max="77" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="78" max="78" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:106" x14ac:dyDescent="0.25">
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
-      <c r="N1" s="8">
+      <c r="N1" s="10">
         <v>63</v>
       </c>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
-      <c r="AA1" s="8" t="s">
+      <c r="AA1" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-      <c r="AH1" s="8"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="10"/>
+      <c r="AH1" s="10"/>
       <c r="AI1" s="1"/>
       <c r="AJ1" s="1"/>
       <c r="AK1" s="1"/>
       <c r="AL1" s="1"/>
       <c r="AM1" s="1"/>
-      <c r="AO1" s="8">
+      <c r="AO1" s="10">
         <v>28</v>
       </c>
-      <c r="AP1" s="8"/>
-      <c r="AQ1" s="8"/>
-      <c r="AR1" s="8"/>
-      <c r="AS1" s="8"/>
-      <c r="AT1" s="8"/>
-      <c r="AU1" s="8"/>
-      <c r="AV1" s="8"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="10"/>
+      <c r="AR1" s="10"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="10"/>
+      <c r="AU1" s="10"/>
+      <c r="AV1" s="10"/>
       <c r="AW1" s="1"/>
       <c r="AX1" s="1"/>
       <c r="AY1" s="1"/>
       <c r="AZ1" s="1"/>
       <c r="BA1" s="1"/>
-      <c r="BB1" s="8" t="s">
+      <c r="BB1" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="BC1" s="8"/>
-      <c r="BD1" s="8"/>
-      <c r="BE1" s="8"/>
-      <c r="BF1" s="8"/>
-      <c r="BG1" s="8"/>
-      <c r="BH1" s="8"/>
-      <c r="BI1" s="8"/>
+      <c r="BC1" s="10"/>
+      <c r="BD1" s="10"/>
+      <c r="BE1" s="10"/>
+      <c r="BF1" s="10"/>
+      <c r="BG1" s="10"/>
+      <c r="BH1" s="10"/>
+      <c r="BI1" s="10"/>
       <c r="BJ1" s="1"/>
       <c r="BK1" s="1"/>
       <c r="BL1" s="1"/>
       <c r="BM1" s="1"/>
       <c r="BN1" s="1"/>
-      <c r="BO1" s="8" t="s">
+      <c r="BO1" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="BP1" s="8"/>
-      <c r="BQ1" s="8"/>
-      <c r="BR1" s="8"/>
-      <c r="BS1" s="8"/>
-      <c r="BT1" s="8"/>
-      <c r="BU1" s="8"/>
-      <c r="BV1" s="8"/>
-      <c r="CB1" s="8" t="s">
+      <c r="BP1" s="10"/>
+      <c r="BQ1" s="10"/>
+      <c r="BR1" s="10"/>
+      <c r="BS1" s="10"/>
+      <c r="BT1" s="10"/>
+      <c r="BU1" s="10"/>
+      <c r="BV1" s="10"/>
+      <c r="CB1" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="CC1" s="8"/>
-      <c r="CD1" s="8"/>
-      <c r="CE1" s="8"/>
-      <c r="CF1" s="8"/>
-      <c r="CG1" s="8"/>
-      <c r="CH1" s="8"/>
-      <c r="CI1" s="8"/>
-      <c r="CP1" s="8" t="s">
+      <c r="CC1" s="10"/>
+      <c r="CD1" s="10"/>
+      <c r="CE1" s="10"/>
+      <c r="CF1" s="10"/>
+      <c r="CG1" s="10"/>
+      <c r="CH1" s="10"/>
+      <c r="CI1" s="10"/>
+      <c r="CP1" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="CQ1" s="8"/>
-      <c r="CR1" s="8"/>
-      <c r="CS1" s="8"/>
-      <c r="CT1" s="8"/>
-      <c r="CU1" s="8"/>
-      <c r="CV1" s="8"/>
-      <c r="CW1" s="8"/>
+      <c r="CQ1" s="10"/>
+      <c r="CR1" s="10"/>
+      <c r="CS1" s="10"/>
+      <c r="CT1" s="10"/>
+      <c r="CU1" s="10"/>
+      <c r="CV1" s="10"/>
+      <c r="CW1" s="10"/>
     </row>
     <row r="2" spans="1:106" x14ac:dyDescent="0.25">
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
-      <c r="AA2" s="8"/>
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="8"/>
-      <c r="AD2" s="8"/>
-      <c r="AE2" s="8"/>
-      <c r="AF2" s="8"/>
-      <c r="AG2" s="8"/>
-      <c r="AH2" s="8"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10"/>
+      <c r="AH2" s="10"/>
       <c r="AI2" s="1"/>
       <c r="AJ2" s="1"/>
       <c r="AK2" s="1"/>
       <c r="AL2" s="1"/>
       <c r="AM2" s="1"/>
-      <c r="AO2" s="8"/>
-      <c r="AP2" s="8"/>
-      <c r="AQ2" s="8"/>
-      <c r="AR2" s="8"/>
-      <c r="AS2" s="8"/>
-      <c r="AT2" s="8"/>
-      <c r="AU2" s="8"/>
-      <c r="AV2" s="8"/>
+      <c r="AO2" s="10"/>
+      <c r="AP2" s="10"/>
+      <c r="AQ2" s="10"/>
+      <c r="AR2" s="10"/>
+      <c r="AS2" s="10"/>
+      <c r="AT2" s="10"/>
+      <c r="AU2" s="10"/>
+      <c r="AV2" s="10"/>
       <c r="AW2" s="1"/>
       <c r="AX2" s="1"/>
       <c r="AY2" s="1"/>
       <c r="AZ2" s="1"/>
       <c r="BA2" s="1"/>
-      <c r="BB2" s="8"/>
-      <c r="BC2" s="8"/>
-      <c r="BD2" s="8"/>
-      <c r="BE2" s="8"/>
-      <c r="BF2" s="8"/>
-      <c r="BG2" s="8"/>
-      <c r="BH2" s="8"/>
-      <c r="BI2" s="8"/>
+      <c r="BB2" s="10"/>
+      <c r="BC2" s="10"/>
+      <c r="BD2" s="10"/>
+      <c r="BE2" s="10"/>
+      <c r="BF2" s="10"/>
+      <c r="BG2" s="10"/>
+      <c r="BH2" s="10"/>
+      <c r="BI2" s="10"/>
       <c r="BJ2" s="1"/>
       <c r="BK2" s="1"/>
       <c r="BL2" s="1"/>
       <c r="BM2" s="1"/>
       <c r="BN2" s="1"/>
-      <c r="BO2" s="8"/>
-      <c r="BP2" s="8"/>
-      <c r="BQ2" s="8"/>
-      <c r="BR2" s="8"/>
-      <c r="BS2" s="8"/>
-      <c r="BT2" s="8"/>
-      <c r="BU2" s="8"/>
-      <c r="BV2" s="8"/>
-      <c r="CB2" s="8"/>
-      <c r="CC2" s="8"/>
-      <c r="CD2" s="8"/>
-      <c r="CE2" s="8"/>
-      <c r="CF2" s="8"/>
-      <c r="CG2" s="8"/>
-      <c r="CH2" s="8"/>
-      <c r="CI2" s="8"/>
-      <c r="CP2" s="8"/>
-      <c r="CQ2" s="8"/>
-      <c r="CR2" s="8"/>
-      <c r="CS2" s="8"/>
-      <c r="CT2" s="8"/>
-      <c r="CU2" s="8"/>
-      <c r="CV2" s="8"/>
-      <c r="CW2" s="8"/>
+      <c r="BO2" s="10"/>
+      <c r="BP2" s="10"/>
+      <c r="BQ2" s="10"/>
+      <c r="BR2" s="10"/>
+      <c r="BS2" s="10"/>
+      <c r="BT2" s="10"/>
+      <c r="BU2" s="10"/>
+      <c r="BV2" s="10"/>
+      <c r="CB2" s="10"/>
+      <c r="CC2" s="10"/>
+      <c r="CD2" s="10"/>
+      <c r="CE2" s="10"/>
+      <c r="CF2" s="10"/>
+      <c r="CG2" s="10"/>
+      <c r="CH2" s="10"/>
+      <c r="CI2" s="10"/>
+      <c r="CP2" s="10"/>
+      <c r="CQ2" s="10"/>
+      <c r="CR2" s="10"/>
+      <c r="CS2" s="10"/>
+      <c r="CT2" s="10"/>
+      <c r="CU2" s="10"/>
+      <c r="CV2" s="10"/>
+      <c r="CW2" s="10"/>
     </row>
     <row r="3" spans="1:106" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -7428,6 +7473,42 @@
         <v>71</v>
       </c>
       <c r="CM6" t="s">
+        <v>72</v>
+      </c>
+      <c r="CP6" t="s">
+        <v>64</v>
+      </c>
+      <c r="CQ6" t="s">
+        <v>59</v>
+      </c>
+      <c r="CR6" t="s">
+        <v>60</v>
+      </c>
+      <c r="CS6" t="s">
+        <v>61</v>
+      </c>
+      <c r="CT6" t="s">
+        <v>66</v>
+      </c>
+      <c r="CU6" t="s">
+        <v>67</v>
+      </c>
+      <c r="CV6" t="s">
+        <v>63</v>
+      </c>
+      <c r="CW6" t="s">
+        <v>62</v>
+      </c>
+      <c r="CX6" t="s">
+        <v>69</v>
+      </c>
+      <c r="CY6" t="s">
+        <v>70</v>
+      </c>
+      <c r="CZ6" t="s">
+        <v>71</v>
+      </c>
+      <c r="DA6" t="s">
         <v>72</v>
       </c>
     </row>
@@ -7586,7 +7667,48 @@
       <c r="CN7" t="s">
         <v>117</v>
       </c>
-      <c r="CU7" s="5"/>
+      <c r="CP7" t="s">
+        <v>65</v>
+      </c>
+      <c r="CQ7" t="s">
+        <v>68</v>
+      </c>
+      <c r="CR7" t="s">
+        <v>122</v>
+      </c>
+      <c r="CS7">
+        <v>18000</v>
+      </c>
+      <c r="CT7">
+        <f>CV7/CS7</f>
+        <v>0.48372222222222222</v>
+      </c>
+      <c r="CU7" s="5">
+        <f>1-CT7</f>
+        <v>0.51627777777777784</v>
+      </c>
+      <c r="CV7">
+        <v>8707</v>
+      </c>
+      <c r="CW7">
+        <f>CS7-CV7</f>
+        <v>9293</v>
+      </c>
+      <c r="CX7">
+        <v>20.23</v>
+      </c>
+      <c r="CY7">
+        <v>20.02</v>
+      </c>
+      <c r="CZ7">
+        <v>18.63</v>
+      </c>
+      <c r="DA7">
+        <v>18.760000000000002</v>
+      </c>
+      <c r="DB7" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="9" spans="1:106" x14ac:dyDescent="0.25">
       <c r="N9" t="s">

</xml_diff>